<commit_message>
Reclassify per category standards2: remove G4, redistribute to G1/G2/G3
</commit_message>
<xml_diff>
--- a/dataset2026.xlsx
+++ b/dataset2026.xlsx
@@ -4820,7 +4820,7 @@
         <v>-1</v>
       </c>
       <c r="HV6">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="HX6">
         <v>6</v>
@@ -6065,7 +6065,7 @@
         <v>1</v>
       </c>
       <c r="HX9">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="HZ9">
         <v>1</v>
@@ -8145,10 +8145,10 @@
         <v>-1</v>
       </c>
       <c r="HU14">
-        <v>4</v>
+        <v>1</v>
       </c>
       <c r="HV14">
-        <v>4</v>
+        <v>1</v>
       </c>
       <c r="HW14">
         <v>2</v>
@@ -8594,10 +8594,10 @@
         <v>-1</v>
       </c>
       <c r="HU15">
-        <v>4</v>
+        <v>1</v>
       </c>
       <c r="HV15">
-        <v>4</v>
+        <v>1</v>
       </c>
       <c r="HW15">
         <v>2</v>
@@ -9043,10 +9043,10 @@
         <v>-1</v>
       </c>
       <c r="HU16">
-        <v>4</v>
+        <v>1</v>
       </c>
       <c r="HV16">
-        <v>4</v>
+        <v>1</v>
       </c>
       <c r="HW16">
         <v>2</v>
@@ -11027,7 +11027,7 @@
         <v>-1</v>
       </c>
       <c r="HU21">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="HW21">
         <v>2</v>
@@ -13089,7 +13089,7 @@
         <v>2</v>
       </c>
       <c r="HV26">
-        <v>4</v>
+        <v>1</v>
       </c>
       <c r="HW26">
         <v>3</v>
@@ -13538,7 +13538,7 @@
         <v>2</v>
       </c>
       <c r="HV27">
-        <v>4</v>
+        <v>1</v>
       </c>
       <c r="HW27">
         <v>3</v>
@@ -13987,7 +13987,7 @@
         <v>2</v>
       </c>
       <c r="HV28">
-        <v>4</v>
+        <v>1</v>
       </c>
       <c r="HW28">
         <v>2</v>
@@ -14436,13 +14436,13 @@
         <v>2</v>
       </c>
       <c r="HV29">
-        <v>4</v>
+        <v>1</v>
       </c>
       <c r="HW29">
         <v>3</v>
       </c>
       <c r="HX29">
-        <v>3</v>
+        <v>6</v>
       </c>
       <c r="HY29">
         <v>1</v>
@@ -14885,7 +14885,7 @@
         <v>2</v>
       </c>
       <c r="HV30">
-        <v>4</v>
+        <v>1</v>
       </c>
       <c r="HW30">
         <v>2</v>
@@ -15334,7 +15334,7 @@
         <v>2</v>
       </c>
       <c r="HV31">
-        <v>4</v>
+        <v>1</v>
       </c>
       <c r="HW31">
         <v>4</v>
@@ -17100,7 +17100,7 @@
         <v>2</v>
       </c>
       <c r="HV35">
-        <v>4</v>
+        <v>1</v>
       </c>
       <c r="HW35">
         <v>2</v>
@@ -17549,7 +17549,7 @@
         <v>2</v>
       </c>
       <c r="HV36">
-        <v>4</v>
+        <v>1</v>
       </c>
       <c r="HW36">
         <v>3</v>
@@ -17998,7 +17998,7 @@
         <v>2</v>
       </c>
       <c r="HV37">
-        <v>4</v>
+        <v>1</v>
       </c>
       <c r="HW37">
         <v>2</v>
@@ -20015,7 +20015,7 @@
         <v>1</v>
       </c>
       <c r="HV42">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="HW42">
         <v>3</v>
@@ -22242,10 +22242,10 @@
         <v>-1</v>
       </c>
       <c r="HU47">
-        <v>4</v>
+        <v>2</v>
       </c>
       <c r="HV47">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="HW47">
         <v>3</v>
@@ -22691,10 +22691,10 @@
         <v>-1</v>
       </c>
       <c r="HU48">
-        <v>4</v>
+        <v>2</v>
       </c>
       <c r="HV48">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="HW48">
         <v>2</v>
@@ -23140,7 +23140,7 @@
         <v>-1</v>
       </c>
       <c r="HU49">
-        <v>4</v>
+        <v>2</v>
       </c>
       <c r="HW49">
         <v>2</v>
@@ -23577,7 +23577,7 @@
         <v>-1</v>
       </c>
       <c r="HU50">
-        <v>4</v>
+        <v>1</v>
       </c>
       <c r="HV50">
         <v>3</v>
@@ -24023,7 +24023,7 @@
         <v>-1</v>
       </c>
       <c r="HU51">
-        <v>4</v>
+        <v>1</v>
       </c>
       <c r="HV51">
         <v>3</v>
@@ -24469,7 +24469,7 @@
         <v>-1</v>
       </c>
       <c r="HU52">
-        <v>4</v>
+        <v>1</v>
       </c>
       <c r="HV52">
         <v>3</v>
@@ -24906,7 +24906,7 @@
         <v>2</v>
       </c>
       <c r="HW53">
-        <v>3</v>
+        <v>6</v>
       </c>
       <c r="HY53">
         <v>1</v>
@@ -26145,7 +26145,7 @@
         <v>1</v>
       </c>
       <c r="HU56">
-        <v>4</v>
+        <v>1</v>
       </c>
       <c r="HV56">
         <v>2</v>
@@ -27022,7 +27022,7 @@
         <v>1</v>
       </c>
       <c r="HU58">
-        <v>4</v>
+        <v>1</v>
       </c>
       <c r="HV58">
         <v>2</v>
@@ -28809,7 +28809,7 @@
         <v>1</v>
       </c>
       <c r="HV62">
-        <v>4</v>
+        <v>1</v>
       </c>
       <c r="HW62">
         <v>3</v>
@@ -29255,7 +29255,7 @@
         <v>1</v>
       </c>
       <c r="HV63">
-        <v>4</v>
+        <v>1</v>
       </c>
       <c r="HW63">
         <v>4</v>
@@ -29701,7 +29701,7 @@
         <v>1</v>
       </c>
       <c r="HV64">
-        <v>4</v>
+        <v>1</v>
       </c>
       <c r="HW64">
         <v>2</v>
@@ -31485,7 +31485,7 @@
         <v>3</v>
       </c>
       <c r="HV68">
-        <v>4</v>
+        <v>1</v>
       </c>
       <c r="HW68">
         <v>3</v>
@@ -32362,13 +32362,13 @@
         <v>3</v>
       </c>
       <c r="HV70">
-        <v>4</v>
+        <v>1</v>
       </c>
       <c r="HW70">
         <v>2</v>
       </c>
       <c r="HX70">
-        <v>5</v>
+        <v>2</v>
       </c>
       <c r="HY70">
         <v>1</v>
@@ -32808,7 +32808,7 @@
         <v>2</v>
       </c>
       <c r="HV71">
-        <v>4</v>
+        <v>1</v>
       </c>
       <c r="HW71">
         <v>6</v>
@@ -33254,7 +33254,7 @@
         <v>2</v>
       </c>
       <c r="HV72">
-        <v>4</v>
+        <v>1</v>
       </c>
       <c r="HW72">
         <v>3</v>
@@ -33697,7 +33697,7 @@
         <v>0</v>
       </c>
       <c r="HV73">
-        <v>4</v>
+        <v>1</v>
       </c>
       <c r="HW73">
         <v>2</v>
@@ -40308,7 +40308,7 @@
         <v>2</v>
       </c>
       <c r="HV89">
-        <v>4</v>
+        <v>1</v>
       </c>
       <c r="HW89">
         <v>3</v>
@@ -40754,7 +40754,7 @@
         <v>2</v>
       </c>
       <c r="HV90">
-        <v>4</v>
+        <v>1</v>
       </c>
       <c r="HW90">
         <v>3</v>
@@ -41200,7 +41200,7 @@
         <v>2</v>
       </c>
       <c r="HV91">
-        <v>4</v>
+        <v>1</v>
       </c>
       <c r="HW91">
         <v>2</v>
@@ -41649,7 +41649,7 @@
         <v>1</v>
       </c>
       <c r="HV92">
-        <v>4</v>
+        <v>1</v>
       </c>
       <c r="HW92">
         <v>3</v>
@@ -42098,7 +42098,7 @@
         <v>1</v>
       </c>
       <c r="HV93">
-        <v>4</v>
+        <v>1</v>
       </c>
       <c r="HW93">
         <v>2</v>
@@ -42547,7 +42547,7 @@
         <v>1</v>
       </c>
       <c r="HV94">
-        <v>4</v>
+        <v>1</v>
       </c>
       <c r="HW94">
         <v>2</v>
@@ -44328,7 +44328,7 @@
         <v>-1</v>
       </c>
       <c r="HU98">
-        <v>4</v>
+        <v>1</v>
       </c>
       <c r="HW98">
         <v>2</v>
@@ -44741,7 +44741,7 @@
         <v>-1</v>
       </c>
       <c r="HU99">
-        <v>4</v>
+        <v>1</v>
       </c>
       <c r="HW99">
         <v>4</v>
@@ -45154,7 +45154,7 @@
         <v>-1</v>
       </c>
       <c r="HU100">
-        <v>4</v>
+        <v>1</v>
       </c>
       <c r="HW100">
         <v>2</v>
@@ -45579,10 +45579,10 @@
         <v>0</v>
       </c>
       <c r="HU101">
-        <v>4</v>
+        <v>1</v>
       </c>
       <c r="HV101">
-        <v>4</v>
+        <v>1</v>
       </c>
       <c r="HW101">
         <v>2</v>
@@ -46028,10 +46028,10 @@
         <v>1</v>
       </c>
       <c r="HU102">
-        <v>4</v>
+        <v>1</v>
       </c>
       <c r="HV102">
-        <v>4</v>
+        <v>1</v>
       </c>
       <c r="HW102">
         <v>3</v>
@@ -46477,10 +46477,10 @@
         <v>1</v>
       </c>
       <c r="HU103">
-        <v>4</v>
+        <v>1</v>
       </c>
       <c r="HV103">
-        <v>4</v>
+        <v>1</v>
       </c>
       <c r="HW103">
         <v>2</v>
@@ -46929,7 +46929,7 @@
         <v>2</v>
       </c>
       <c r="HV104">
-        <v>4</v>
+        <v>1</v>
       </c>
       <c r="HW104">
         <v>3</v>
@@ -47378,7 +47378,7 @@
         <v>2</v>
       </c>
       <c r="HV105">
-        <v>4</v>
+        <v>1</v>
       </c>
       <c r="HW105">
         <v>2</v>
@@ -47827,7 +47827,7 @@
         <v>2</v>
       </c>
       <c r="HV106">
-        <v>4</v>
+        <v>1</v>
       </c>
       <c r="HW106">
         <v>2</v>
@@ -48276,7 +48276,7 @@
         <v>2</v>
       </c>
       <c r="HV107">
-        <v>4</v>
+        <v>1</v>
       </c>
       <c r="HW107">
         <v>2</v>
@@ -48725,7 +48725,7 @@
         <v>2</v>
       </c>
       <c r="HV108">
-        <v>4</v>
+        <v>1</v>
       </c>
       <c r="HW108">
         <v>3</v>
@@ -49174,7 +49174,7 @@
         <v>2</v>
       </c>
       <c r="HV109">
-        <v>4</v>
+        <v>1</v>
       </c>
       <c r="HW109">
         <v>3</v>
@@ -52119,7 +52119,7 @@
         <v>2</v>
       </c>
       <c r="HV116">
-        <v>4</v>
+        <v>1</v>
       </c>
       <c r="HW116">
         <v>3</v>
@@ -52568,7 +52568,7 @@
         <v>2</v>
       </c>
       <c r="HV117">
-        <v>4</v>
+        <v>1</v>
       </c>
       <c r="HW117">
         <v>2</v>
@@ -53017,7 +53017,7 @@
         <v>2</v>
       </c>
       <c r="HV118">
-        <v>4</v>
+        <v>1</v>
       </c>
       <c r="HW118">
         <v>2</v>
@@ -53466,7 +53466,7 @@
         <v>2</v>
       </c>
       <c r="HV119">
-        <v>4</v>
+        <v>1</v>
       </c>
       <c r="HW119">
         <v>3</v>
@@ -53915,7 +53915,7 @@
         <v>2</v>
       </c>
       <c r="HV120">
-        <v>4</v>
+        <v>1</v>
       </c>
       <c r="HW120">
         <v>2</v>
@@ -54364,7 +54364,7 @@
         <v>2</v>
       </c>
       <c r="HV121">
-        <v>4</v>
+        <v>1</v>
       </c>
       <c r="HW121">
         <v>1</v>
@@ -57833,7 +57833,7 @@
         <v>2</v>
       </c>
       <c r="HV129">
-        <v>4</v>
+        <v>1</v>
       </c>
       <c r="HW129">
         <v>3</v>
@@ -58282,7 +58282,7 @@
         <v>2</v>
       </c>
       <c r="HV130">
-        <v>4</v>
+        <v>1</v>
       </c>
       <c r="HW130">
         <v>3</v>
@@ -58722,7 +58722,7 @@
         <v>-1</v>
       </c>
       <c r="HU131">
-        <v>4</v>
+        <v>1</v>
       </c>
       <c r="HW131">
         <v>2</v>
@@ -59141,7 +59141,7 @@
         <v>-1</v>
       </c>
       <c r="HU132">
-        <v>4</v>
+        <v>1</v>
       </c>
       <c r="HW132">
         <v>2</v>
@@ -59560,10 +59560,10 @@
         <v>-1</v>
       </c>
       <c r="HU133">
-        <v>4</v>
+        <v>1</v>
       </c>
       <c r="HW133">
-        <v>3</v>
+        <v>6</v>
       </c>
       <c r="HY133">
         <v>1</v>
@@ -60401,7 +60401,7 @@
         <v>3</v>
       </c>
       <c r="HX135">
-        <v>5</v>
+        <v>2</v>
       </c>
       <c r="HZ135">
         <v>1</v>
@@ -60820,7 +60820,7 @@
         <v>3</v>
       </c>
       <c r="HX136">
-        <v>5</v>
+        <v>2</v>
       </c>
       <c r="HZ136">
         <v>1</v>
@@ -62388,7 +62388,7 @@
         <v>1</v>
       </c>
       <c r="HU140">
-        <v>4</v>
+        <v>1</v>
       </c>
       <c r="HV140">
         <v>2</v>
@@ -62834,7 +62834,7 @@
         <v>1</v>
       </c>
       <c r="HU141">
-        <v>4</v>
+        <v>1</v>
       </c>
       <c r="HV141">
         <v>2</v>
@@ -63280,7 +63280,7 @@
         <v>0</v>
       </c>
       <c r="HU142">
-        <v>4</v>
+        <v>1</v>
       </c>
       <c r="HV142">
         <v>2</v>
@@ -65064,10 +65064,10 @@
         <v>-1</v>
       </c>
       <c r="HU146">
-        <v>4</v>
+        <v>1</v>
       </c>
       <c r="HV146">
-        <v>4</v>
+        <v>1</v>
       </c>
       <c r="HW146">
         <v>3</v>
@@ -65510,10 +65510,10 @@
         <v>-1</v>
       </c>
       <c r="HU147">
-        <v>4</v>
+        <v>1</v>
       </c>
       <c r="HV147">
-        <v>4</v>
+        <v>1</v>
       </c>
       <c r="HW147">
         <v>2</v>
@@ -65956,10 +65956,10 @@
         <v>-1</v>
       </c>
       <c r="HU148">
-        <v>4</v>
+        <v>1</v>
       </c>
       <c r="HV148">
-        <v>4</v>
+        <v>1</v>
       </c>
       <c r="HW148">
         <v>2</v>
@@ -68952,10 +68952,10 @@
         <v>3</v>
       </c>
       <c r="HV155">
-        <v>4</v>
+        <v>1</v>
       </c>
       <c r="HW155">
-        <v>3</v>
+        <v>6</v>
       </c>
       <c r="HX155">
         <v>2</v>
@@ -69398,7 +69398,7 @@
         <v>3</v>
       </c>
       <c r="HV156">
-        <v>4</v>
+        <v>1</v>
       </c>
       <c r="HW156">
         <v>3</v>
@@ -70296,10 +70296,10 @@
         <v>3</v>
       </c>
       <c r="HV158">
-        <v>4</v>
+        <v>1</v>
       </c>
       <c r="HW158">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="HX158">
         <v>3</v>
@@ -70778,7 +70778,7 @@
         <v>3</v>
       </c>
       <c r="HV159">
-        <v>4</v>
+        <v>1</v>
       </c>
       <c r="HW159">
         <v>2</v>
@@ -71260,7 +71260,7 @@
         <v>3</v>
       </c>
       <c r="HV160">
-        <v>4</v>
+        <v>1</v>
       </c>
       <c r="HW160">
         <v>2</v>
@@ -74361,10 +74361,10 @@
         <v>2</v>
       </c>
       <c r="HV167">
-        <v>4</v>
+        <v>1</v>
       </c>
       <c r="HW167">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="HX167">
         <v>1</v>
@@ -74807,7 +74807,7 @@
         <v>2</v>
       </c>
       <c r="HV168">
-        <v>4</v>
+        <v>1</v>
       </c>
       <c r="HW168">
         <v>2</v>
@@ -75253,7 +75253,7 @@
         <v>2</v>
       </c>
       <c r="HV169">
-        <v>4</v>
+        <v>1</v>
       </c>
       <c r="HW169">
         <v>2</v>
@@ -75699,7 +75699,7 @@
         <v>3</v>
       </c>
       <c r="HV170">
-        <v>4</v>
+        <v>2</v>
       </c>
       <c r="HW170">
         <v>2</v>
@@ -76145,7 +76145,7 @@
         <v>3</v>
       </c>
       <c r="HV171">
-        <v>4</v>
+        <v>2</v>
       </c>
       <c r="HW171">
         <v>3</v>
@@ -78249,10 +78249,10 @@
         <v>1</v>
       </c>
       <c r="HU176">
-        <v>4</v>
+        <v>1</v>
       </c>
       <c r="HV176">
-        <v>4</v>
+        <v>1</v>
       </c>
       <c r="HW176">
         <v>2</v>
@@ -78695,7 +78695,7 @@
         <v>0</v>
       </c>
       <c r="HU177">
-        <v>4</v>
+        <v>1</v>
       </c>
       <c r="HW177">
         <v>2</v>
@@ -79126,10 +79126,10 @@
         <v>1</v>
       </c>
       <c r="HU178">
-        <v>4</v>
+        <v>1</v>
       </c>
       <c r="HV178">
-        <v>4</v>
+        <v>1</v>
       </c>
       <c r="HW178">
         <v>3</v>
@@ -79575,7 +79575,7 @@
         <v>2</v>
       </c>
       <c r="HV179">
-        <v>4</v>
+        <v>1</v>
       </c>
       <c r="HW179">
         <v>2</v>
@@ -80021,7 +80021,7 @@
         <v>2</v>
       </c>
       <c r="HV180">
-        <v>4</v>
+        <v>1</v>
       </c>
       <c r="HW180">
         <v>6</v>
@@ -80467,7 +80467,7 @@
         <v>2</v>
       </c>
       <c r="HV181">
-        <v>4</v>
+        <v>1</v>
       </c>
       <c r="HW181">
         <v>3</v>
@@ -80910,7 +80910,7 @@
         <v>-1</v>
       </c>
       <c r="HV182">
-        <v>4</v>
+        <v>1</v>
       </c>
       <c r="HX182">
         <v>3</v>
@@ -81772,7 +81772,7 @@
         <v>-1</v>
       </c>
       <c r="HV184">
-        <v>4</v>
+        <v>1</v>
       </c>
       <c r="HX184">
         <v>2</v>

</xml_diff>

<commit_message>
Reassign individual_type1/2 with clean I1-I7 to 7-type mapping, TR=1 no Type 4
</commit_message>
<xml_diff>
--- a/dataset2026.xlsx
+++ b/dataset2026.xlsx
@@ -784,12 +784,6 @@
     <t>chat_type2</t>
   </si>
   <si>
-    <t>individual_type1</t>
-  </si>
-  <si>
-    <t>individual_type2</t>
-  </si>
-  <si>
     <t>third_party_group1</t>
   </si>
   <si>
@@ -806,6 +800,12 @@
   </si>
   <si>
     <t>discuss2</t>
+  </si>
+  <si>
+    <t>individual_type1</t>
+  </si>
+  <si>
+    <t>individual_type2</t>
   </si>
   <si>
     <t>2023.12.14</t>
@@ -3330,19 +3330,19 @@
         <v>1</v>
       </c>
       <c r="IW2">
+        <v>1</v>
+      </c>
+      <c r="IY2">
+        <v>1</v>
+      </c>
+      <c r="JA2">
+        <v>1</v>
+      </c>
+      <c r="JB2">
+        <v>0</v>
+      </c>
+      <c r="JC2">
         <v>6</v>
-      </c>
-      <c r="IY2">
-        <v>1</v>
-      </c>
-      <c r="JA2">
-        <v>1</v>
-      </c>
-      <c r="JC2">
-        <v>1</v>
-      </c>
-      <c r="JD2">
-        <v>0</v>
       </c>
     </row>
     <row r="3" spans="1:264">
@@ -3779,7 +3779,7 @@
         <v>1</v>
       </c>
       <c r="IW3">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="IY3">
         <v>1</v>
@@ -3787,11 +3787,11 @@
       <c r="JA3">
         <v>1</v>
       </c>
+      <c r="JB3">
+        <v>0</v>
+      </c>
       <c r="JC3">
-        <v>1</v>
-      </c>
-      <c r="JD3">
-        <v>0</v>
+        <v>2</v>
       </c>
     </row>
     <row r="4" spans="1:264">
@@ -4236,11 +4236,11 @@
       <c r="JA4">
         <v>1</v>
       </c>
+      <c r="JB4">
+        <v>0</v>
+      </c>
       <c r="JC4">
         <v>1</v>
-      </c>
-      <c r="JD4">
-        <v>0</v>
       </c>
     </row>
     <row r="5" spans="1:264">
@@ -4658,10 +4658,10 @@
       <c r="IN5">
         <v>2</v>
       </c>
-      <c r="JC5">
-        <v>0</v>
-      </c>
-      <c r="JD5">
+      <c r="JA5">
+        <v>0</v>
+      </c>
+      <c r="JB5">
         <v>0</v>
       </c>
     </row>
@@ -5105,19 +5105,19 @@
         <v>6</v>
       </c>
       <c r="IX6">
+        <v>1</v>
+      </c>
+      <c r="IZ6">
+        <v>1</v>
+      </c>
+      <c r="JA6">
+        <v>0</v>
+      </c>
+      <c r="JB6">
+        <v>1</v>
+      </c>
+      <c r="JD6">
         <v>7</v>
-      </c>
-      <c r="IZ6">
-        <v>1</v>
-      </c>
-      <c r="JB6">
-        <v>1</v>
-      </c>
-      <c r="JC6">
-        <v>0</v>
-      </c>
-      <c r="JD6">
-        <v>1</v>
       </c>
     </row>
     <row r="7" spans="1:264">
@@ -5535,10 +5535,10 @@
       <c r="IN7">
         <v>3</v>
       </c>
-      <c r="JC7">
-        <v>0</v>
-      </c>
-      <c r="JD7">
+      <c r="JA7">
+        <v>0</v>
+      </c>
+      <c r="JB7">
         <v>0</v>
       </c>
     </row>
@@ -5982,19 +5982,19 @@
         <v>3</v>
       </c>
       <c r="IX8">
+        <v>1</v>
+      </c>
+      <c r="IZ8">
+        <v>1</v>
+      </c>
+      <c r="JA8">
+        <v>0</v>
+      </c>
+      <c r="JB8">
+        <v>1</v>
+      </c>
+      <c r="JD8">
         <v>7</v>
-      </c>
-      <c r="IZ8">
-        <v>1</v>
-      </c>
-      <c r="JB8">
-        <v>1</v>
-      </c>
-      <c r="JC8">
-        <v>0</v>
-      </c>
-      <c r="JD8">
-        <v>1</v>
       </c>
     </row>
     <row r="9" spans="1:264">
@@ -6437,19 +6437,19 @@
         <v>3</v>
       </c>
       <c r="IX9">
+        <v>1</v>
+      </c>
+      <c r="IZ9">
+        <v>1</v>
+      </c>
+      <c r="JA9">
+        <v>0</v>
+      </c>
+      <c r="JB9">
+        <v>1</v>
+      </c>
+      <c r="JD9">
         <v>6</v>
-      </c>
-      <c r="IZ9">
-        <v>1</v>
-      </c>
-      <c r="JB9">
-        <v>1</v>
-      </c>
-      <c r="JC9">
-        <v>0</v>
-      </c>
-      <c r="JD9">
-        <v>1</v>
       </c>
     </row>
     <row r="10" spans="1:264">
@@ -6892,19 +6892,19 @@
         <v>3</v>
       </c>
       <c r="IX10">
+        <v>1</v>
+      </c>
+      <c r="IZ10">
+        <v>1</v>
+      </c>
+      <c r="JA10">
+        <v>0</v>
+      </c>
+      <c r="JB10">
+        <v>1</v>
+      </c>
+      <c r="JD10">
         <v>6</v>
-      </c>
-      <c r="IZ10">
-        <v>1</v>
-      </c>
-      <c r="JB10">
-        <v>1</v>
-      </c>
-      <c r="JC10">
-        <v>0</v>
-      </c>
-      <c r="JD10">
-        <v>1</v>
       </c>
     </row>
     <row r="11" spans="1:264">
@@ -7349,11 +7349,11 @@
       <c r="JA11">
         <v>1</v>
       </c>
+      <c r="JB11">
+        <v>0</v>
+      </c>
       <c r="JC11">
         <v>1</v>
-      </c>
-      <c r="JD11">
-        <v>0</v>
       </c>
     </row>
     <row r="12" spans="1:264">
@@ -7790,7 +7790,7 @@
         <v>1</v>
       </c>
       <c r="IW12">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="IY12">
         <v>1</v>
@@ -7798,11 +7798,11 @@
       <c r="JA12">
         <v>1</v>
       </c>
+      <c r="JB12">
+        <v>0</v>
+      </c>
       <c r="JC12">
-        <v>1</v>
-      </c>
-      <c r="JD12">
-        <v>0</v>
+        <v>2</v>
       </c>
     </row>
     <row r="13" spans="1:264">
@@ -8239,7 +8239,7 @@
         <v>1</v>
       </c>
       <c r="IW13">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="IY13">
         <v>1</v>
@@ -8247,11 +8247,11 @@
       <c r="JA13">
         <v>1</v>
       </c>
+      <c r="JB13">
+        <v>0</v>
+      </c>
       <c r="JC13">
-        <v>1</v>
-      </c>
-      <c r="JD13">
-        <v>0</v>
+        <v>2</v>
       </c>
     </row>
     <row r="14" spans="1:264">
@@ -8733,28 +8733,28 @@
         <v>5</v>
       </c>
       <c r="IW14">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="IX14">
+        <v>1</v>
+      </c>
+      <c r="IY14">
+        <v>1</v>
+      </c>
+      <c r="IZ14">
+        <v>1</v>
+      </c>
+      <c r="JA14">
+        <v>1</v>
+      </c>
+      <c r="JB14">
+        <v>1</v>
+      </c>
+      <c r="JC14">
+        <v>2</v>
+      </c>
+      <c r="JD14">
         <v>7</v>
-      </c>
-      <c r="IY14">
-        <v>1</v>
-      </c>
-      <c r="IZ14">
-        <v>1</v>
-      </c>
-      <c r="JA14">
-        <v>1</v>
-      </c>
-      <c r="JB14">
-        <v>1</v>
-      </c>
-      <c r="JC14">
-        <v>1</v>
-      </c>
-      <c r="JD14">
-        <v>1</v>
       </c>
     </row>
     <row r="15" spans="1:264">
@@ -9236,10 +9236,10 @@
         <v>5</v>
       </c>
       <c r="IW15">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="IX15">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="IY15">
         <v>1</v>
@@ -9254,10 +9254,10 @@
         <v>1</v>
       </c>
       <c r="JC15">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="JD15">
-        <v>1</v>
+        <v>2</v>
       </c>
     </row>
     <row r="16" spans="1:264">
@@ -9739,7 +9739,7 @@
         <v>5</v>
       </c>
       <c r="IW16">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="IX16">
         <v>1</v>
@@ -9757,7 +9757,7 @@
         <v>1</v>
       </c>
       <c r="JC16">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="JD16">
         <v>1</v>
@@ -10157,10 +10157,10 @@
       <c r="IN17">
         <v>2</v>
       </c>
-      <c r="JC17">
-        <v>0</v>
-      </c>
-      <c r="JD17">
+      <c r="JA17">
+        <v>0</v>
+      </c>
+      <c r="JB17">
         <v>0</v>
       </c>
     </row>
@@ -10558,10 +10558,10 @@
       <c r="IN18">
         <v>2</v>
       </c>
-      <c r="JC18">
-        <v>0</v>
-      </c>
-      <c r="JD18">
+      <c r="JA18">
+        <v>0</v>
+      </c>
+      <c r="JB18">
         <v>0</v>
       </c>
     </row>
@@ -10959,10 +10959,10 @@
       <c r="IN19">
         <v>2</v>
       </c>
-      <c r="JC19">
-        <v>0</v>
-      </c>
-      <c r="JD19">
+      <c r="JA19">
+        <v>0</v>
+      </c>
+      <c r="JB19">
         <v>0</v>
       </c>
     </row>
@@ -11375,10 +11375,10 @@
       <c r="IN20">
         <v>3</v>
       </c>
-      <c r="JC20">
-        <v>0</v>
-      </c>
-      <c r="JD20">
+      <c r="JA20">
+        <v>0</v>
+      </c>
+      <c r="JB20">
         <v>0</v>
       </c>
     </row>
@@ -11816,7 +11816,7 @@
         <v>6</v>
       </c>
       <c r="IW21">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="IY21">
         <v>1</v>
@@ -11824,11 +11824,11 @@
       <c r="JA21">
         <v>1</v>
       </c>
+      <c r="JB21">
+        <v>0</v>
+      </c>
       <c r="JC21">
-        <v>1</v>
-      </c>
-      <c r="JD21">
-        <v>0</v>
+        <v>2</v>
       </c>
     </row>
     <row r="22" spans="1:264">
@@ -12240,10 +12240,10 @@
       <c r="IN22">
         <v>2</v>
       </c>
-      <c r="JC22">
-        <v>0</v>
-      </c>
-      <c r="JD22">
+      <c r="JA22">
+        <v>0</v>
+      </c>
+      <c r="JB22">
         <v>0</v>
       </c>
     </row>
@@ -12678,7 +12678,7 @@
         <v>1</v>
       </c>
       <c r="IW23">
-        <v>4</v>
+        <v>1</v>
       </c>
       <c r="IY23">
         <v>1</v>
@@ -12686,11 +12686,11 @@
       <c r="JA23">
         <v>1</v>
       </c>
+      <c r="JB23">
+        <v>0</v>
+      </c>
       <c r="JC23">
-        <v>1</v>
-      </c>
-      <c r="JD23">
-        <v>0</v>
+        <v>4</v>
       </c>
     </row>
     <row r="24" spans="1:264">
@@ -13127,7 +13127,7 @@
         <v>1</v>
       </c>
       <c r="IW24">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="IY24">
         <v>1</v>
@@ -13135,11 +13135,11 @@
       <c r="JA24">
         <v>1</v>
       </c>
+      <c r="JB24">
+        <v>0</v>
+      </c>
       <c r="JC24">
-        <v>1</v>
-      </c>
-      <c r="JD24">
-        <v>0</v>
+        <v>2</v>
       </c>
     </row>
     <row r="25" spans="1:264">
@@ -13576,19 +13576,19 @@
         <v>1</v>
       </c>
       <c r="IW25">
+        <v>1</v>
+      </c>
+      <c r="IY25">
+        <v>1</v>
+      </c>
+      <c r="JA25">
+        <v>1</v>
+      </c>
+      <c r="JB25">
+        <v>0</v>
+      </c>
+      <c r="JC25">
         <v>7</v>
-      </c>
-      <c r="IY25">
-        <v>1</v>
-      </c>
-      <c r="JA25">
-        <v>1</v>
-      </c>
-      <c r="JC25">
-        <v>1</v>
-      </c>
-      <c r="JD25">
-        <v>0</v>
       </c>
     </row>
     <row r="26" spans="1:264">
@@ -14576,7 +14576,7 @@
         <v>1</v>
       </c>
       <c r="IX27">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="IY27">
         <v>1</v>
@@ -14594,7 +14594,7 @@
         <v>1</v>
       </c>
       <c r="JD27">
-        <v>1</v>
+        <v>2</v>
       </c>
     </row>
     <row r="28" spans="1:264">
@@ -15076,10 +15076,10 @@
         <v>5</v>
       </c>
       <c r="IW28">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="IX28">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="IY28">
         <v>1</v>
@@ -15094,10 +15094,10 @@
         <v>1</v>
       </c>
       <c r="JC28">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="JD28">
-        <v>1</v>
+        <v>2</v>
       </c>
     </row>
     <row r="29" spans="1:264">
@@ -15582,25 +15582,25 @@
         <v>1</v>
       </c>
       <c r="IX29">
+        <v>1</v>
+      </c>
+      <c r="IY29">
+        <v>1</v>
+      </c>
+      <c r="IZ29">
+        <v>1</v>
+      </c>
+      <c r="JA29">
+        <v>1</v>
+      </c>
+      <c r="JB29">
+        <v>1</v>
+      </c>
+      <c r="JC29">
+        <v>1</v>
+      </c>
+      <c r="JD29">
         <v>7</v>
-      </c>
-      <c r="IY29">
-        <v>1</v>
-      </c>
-      <c r="IZ29">
-        <v>1</v>
-      </c>
-      <c r="JA29">
-        <v>1</v>
-      </c>
-      <c r="JB29">
-        <v>1</v>
-      </c>
-      <c r="JC29">
-        <v>1</v>
-      </c>
-      <c r="JD29">
-        <v>1</v>
       </c>
     </row>
     <row r="30" spans="1:264">
@@ -16082,28 +16082,28 @@
         <v>3</v>
       </c>
       <c r="IW30">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="IX30">
+        <v>1</v>
+      </c>
+      <c r="IY30">
+        <v>1</v>
+      </c>
+      <c r="IZ30">
+        <v>1</v>
+      </c>
+      <c r="JA30">
+        <v>1</v>
+      </c>
+      <c r="JB30">
+        <v>1</v>
+      </c>
+      <c r="JC30">
+        <v>2</v>
+      </c>
+      <c r="JD30">
         <v>7</v>
-      </c>
-      <c r="IY30">
-        <v>1</v>
-      </c>
-      <c r="IZ30">
-        <v>1</v>
-      </c>
-      <c r="JA30">
-        <v>1</v>
-      </c>
-      <c r="JB30">
-        <v>1</v>
-      </c>
-      <c r="JC30">
-        <v>1</v>
-      </c>
-      <c r="JD30">
-        <v>1</v>
       </c>
     </row>
     <row r="31" spans="1:264">
@@ -16585,28 +16585,28 @@
         <v>3</v>
       </c>
       <c r="IW31">
+        <v>1</v>
+      </c>
+      <c r="IX31">
+        <v>1</v>
+      </c>
+      <c r="IY31">
+        <v>1</v>
+      </c>
+      <c r="IZ31">
+        <v>1</v>
+      </c>
+      <c r="JA31">
+        <v>1</v>
+      </c>
+      <c r="JB31">
+        <v>1</v>
+      </c>
+      <c r="JC31">
         <v>6</v>
       </c>
-      <c r="IX31">
+      <c r="JD31">
         <v>6</v>
-      </c>
-      <c r="IY31">
-        <v>1</v>
-      </c>
-      <c r="IZ31">
-        <v>1</v>
-      </c>
-      <c r="JA31">
-        <v>1</v>
-      </c>
-      <c r="JB31">
-        <v>1</v>
-      </c>
-      <c r="JC31">
-        <v>1</v>
-      </c>
-      <c r="JD31">
-        <v>1</v>
       </c>
     </row>
     <row r="32" spans="1:264">
@@ -17088,28 +17088,28 @@
         <v>4</v>
       </c>
       <c r="IW32">
-        <v>4</v>
+        <v>1</v>
       </c>
       <c r="IX32">
+        <v>0</v>
+      </c>
+      <c r="IY32">
+        <v>1</v>
+      </c>
+      <c r="IZ32">
+        <v>1</v>
+      </c>
+      <c r="JA32">
+        <v>1</v>
+      </c>
+      <c r="JB32">
+        <v>1</v>
+      </c>
+      <c r="JC32">
+        <v>4</v>
+      </c>
+      <c r="JD32">
         <v>6</v>
-      </c>
-      <c r="IY32">
-        <v>1</v>
-      </c>
-      <c r="IZ32">
-        <v>0</v>
-      </c>
-      <c r="JA32">
-        <v>1</v>
-      </c>
-      <c r="JB32">
-        <v>1</v>
-      </c>
-      <c r="JC32">
-        <v>1</v>
-      </c>
-      <c r="JD32">
-        <v>1</v>
       </c>
     </row>
     <row r="33" spans="1:264">
@@ -17542,10 +17542,10 @@
       <c r="IN33">
         <v>2</v>
       </c>
-      <c r="JC33">
-        <v>0</v>
-      </c>
-      <c r="JD33">
+      <c r="JA33">
+        <v>0</v>
+      </c>
+      <c r="JB33">
         <v>0</v>
       </c>
     </row>
@@ -18028,16 +18028,16 @@
         <v>4</v>
       </c>
       <c r="IW34">
-        <v>4</v>
+        <v>1</v>
       </c>
       <c r="IX34">
-        <v>2</v>
+        <v>0</v>
       </c>
       <c r="IY34">
         <v>1</v>
       </c>
       <c r="IZ34">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="JA34">
         <v>1</v>
@@ -18046,10 +18046,10 @@
         <v>1</v>
       </c>
       <c r="JC34">
-        <v>1</v>
+        <v>4</v>
       </c>
       <c r="JD34">
-        <v>1</v>
+        <v>2</v>
       </c>
     </row>
     <row r="35" spans="1:264">
@@ -18531,10 +18531,10 @@
         <v>1</v>
       </c>
       <c r="IW35">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="IX35">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="IY35">
         <v>1</v>
@@ -18549,10 +18549,10 @@
         <v>1</v>
       </c>
       <c r="JC35">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="JD35">
-        <v>1</v>
+        <v>2</v>
       </c>
     </row>
     <row r="36" spans="1:264">
@@ -19034,10 +19034,10 @@
         <v>1</v>
       </c>
       <c r="IW36">
-        <v>3</v>
+        <v>1</v>
       </c>
       <c r="IX36">
-        <v>3</v>
+        <v>1</v>
       </c>
       <c r="IY36">
         <v>1</v>
@@ -19052,10 +19052,10 @@
         <v>1</v>
       </c>
       <c r="JC36">
-        <v>1</v>
+        <v>3</v>
       </c>
       <c r="JD36">
-        <v>1</v>
+        <v>3</v>
       </c>
     </row>
     <row r="37" spans="1:264">
@@ -19537,10 +19537,10 @@
         <v>1</v>
       </c>
       <c r="IW37">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="IX37">
-        <v>3</v>
+        <v>1</v>
       </c>
       <c r="IY37">
         <v>1</v>
@@ -19555,10 +19555,10 @@
         <v>1</v>
       </c>
       <c r="JC37">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="JD37">
-        <v>1</v>
+        <v>3</v>
       </c>
     </row>
     <row r="38" spans="1:264">
@@ -19955,10 +19955,10 @@
       <c r="IN38">
         <v>2</v>
       </c>
-      <c r="JC38">
-        <v>0</v>
-      </c>
-      <c r="JD38">
+      <c r="JA38">
+        <v>0</v>
+      </c>
+      <c r="JB38">
         <v>0</v>
       </c>
     </row>
@@ -20356,10 +20356,10 @@
       <c r="IN39">
         <v>2</v>
       </c>
-      <c r="JC39">
-        <v>0</v>
-      </c>
-      <c r="JD39">
+      <c r="JA39">
+        <v>0</v>
+      </c>
+      <c r="JB39">
         <v>0</v>
       </c>
     </row>
@@ -20757,10 +20757,10 @@
       <c r="IN40">
         <v>2</v>
       </c>
-      <c r="JC40">
-        <v>0</v>
-      </c>
-      <c r="JD40">
+      <c r="JA40">
+        <v>0</v>
+      </c>
+      <c r="JB40">
         <v>0</v>
       </c>
     </row>
@@ -21194,10 +21194,10 @@
       <c r="IN41">
         <v>2</v>
       </c>
-      <c r="JC41">
-        <v>0</v>
-      </c>
-      <c r="JD41">
+      <c r="JA41">
+        <v>0</v>
+      </c>
+      <c r="JB41">
         <v>0</v>
       </c>
     </row>
@@ -21680,28 +21680,28 @@
         <v>6</v>
       </c>
       <c r="IW42">
-        <v>4</v>
+        <v>1</v>
       </c>
       <c r="IX42">
+        <v>1</v>
+      </c>
+      <c r="IY42">
+        <v>1</v>
+      </c>
+      <c r="IZ42">
+        <v>1</v>
+      </c>
+      <c r="JA42">
+        <v>1</v>
+      </c>
+      <c r="JB42">
+        <v>1</v>
+      </c>
+      <c r="JC42">
+        <v>4</v>
+      </c>
+      <c r="JD42">
         <v>5</v>
-      </c>
-      <c r="IY42">
-        <v>1</v>
-      </c>
-      <c r="IZ42">
-        <v>1</v>
-      </c>
-      <c r="JA42">
-        <v>1</v>
-      </c>
-      <c r="JB42">
-        <v>1</v>
-      </c>
-      <c r="JC42">
-        <v>1</v>
-      </c>
-      <c r="JD42">
-        <v>1</v>
       </c>
     </row>
     <row r="43" spans="1:264">
@@ -22159,7 +22159,7 @@
         <v>5</v>
       </c>
       <c r="IW43">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="IY43">
         <v>1</v>
@@ -22167,11 +22167,11 @@
       <c r="JA43">
         <v>1</v>
       </c>
+      <c r="JB43">
+        <v>0</v>
+      </c>
       <c r="JC43">
-        <v>1</v>
-      </c>
-      <c r="JD43">
-        <v>0</v>
+        <v>2</v>
       </c>
     </row>
     <row r="44" spans="1:264">
@@ -22653,10 +22653,10 @@
         <v>3</v>
       </c>
       <c r="IW44">
-        <v>3</v>
+        <v>1</v>
       </c>
       <c r="IX44">
-        <v>3</v>
+        <v>1</v>
       </c>
       <c r="IY44">
         <v>1</v>
@@ -22671,10 +22671,10 @@
         <v>1</v>
       </c>
       <c r="JC44">
-        <v>1</v>
+        <v>3</v>
       </c>
       <c r="JD44">
-        <v>1</v>
+        <v>3</v>
       </c>
     </row>
     <row r="45" spans="1:264">
@@ -23156,10 +23156,10 @@
         <v>3</v>
       </c>
       <c r="IW45">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="IX45">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="IY45">
         <v>1</v>
@@ -23174,10 +23174,10 @@
         <v>1</v>
       </c>
       <c r="JC45">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="JD45">
-        <v>1</v>
+        <v>2</v>
       </c>
     </row>
     <row r="46" spans="1:264">
@@ -23659,10 +23659,10 @@
         <v>3</v>
       </c>
       <c r="IW46">
-        <v>4</v>
+        <v>1</v>
       </c>
       <c r="IX46">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="IY46">
         <v>1</v>
@@ -23677,10 +23677,10 @@
         <v>1</v>
       </c>
       <c r="JC46">
-        <v>1</v>
+        <v>4</v>
       </c>
       <c r="JD46">
-        <v>1</v>
+        <v>2</v>
       </c>
     </row>
     <row r="47" spans="1:264">
@@ -24162,28 +24162,28 @@
         <v>1</v>
       </c>
       <c r="IW47">
-        <v>3</v>
+        <v>1</v>
       </c>
       <c r="IX47">
+        <v>1</v>
+      </c>
+      <c r="IY47">
+        <v>1</v>
+      </c>
+      <c r="IZ47">
+        <v>1</v>
+      </c>
+      <c r="JA47">
+        <v>1</v>
+      </c>
+      <c r="JB47">
+        <v>1</v>
+      </c>
+      <c r="JC47">
+        <v>3</v>
+      </c>
+      <c r="JD47">
         <v>5</v>
-      </c>
-      <c r="IY47">
-        <v>1</v>
-      </c>
-      <c r="IZ47">
-        <v>1</v>
-      </c>
-      <c r="JA47">
-        <v>1</v>
-      </c>
-      <c r="JB47">
-        <v>1</v>
-      </c>
-      <c r="JC47">
-        <v>1</v>
-      </c>
-      <c r="JD47">
-        <v>1</v>
       </c>
     </row>
     <row r="48" spans="1:264">
@@ -24665,10 +24665,10 @@
         <v>1</v>
       </c>
       <c r="IW48">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="IX48">
-        <v>3</v>
+        <v>1</v>
       </c>
       <c r="IY48">
         <v>1</v>
@@ -24683,10 +24683,10 @@
         <v>1</v>
       </c>
       <c r="JC48">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="JD48">
-        <v>1</v>
+        <v>3</v>
       </c>
     </row>
     <row r="49" spans="1:264">
@@ -25150,25 +25150,25 @@
         <v>3</v>
       </c>
       <c r="IW49">
-        <v>2</v>
-      </c>
-      <c r="IX49">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="IY49">
         <v>1</v>
       </c>
+      <c r="IZ49">
+        <v>1</v>
+      </c>
       <c r="JA49">
         <v>1</v>
       </c>
       <c r="JB49">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="JC49">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="JD49">
-        <v>0</v>
+        <v>2</v>
       </c>
     </row>
     <row r="50" spans="1:264">
@@ -25647,7 +25647,7 @@
         <v>3</v>
       </c>
       <c r="IW50">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="IX50">
         <v>1</v>
@@ -25665,7 +25665,7 @@
         <v>1</v>
       </c>
       <c r="JC50">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="JD50">
         <v>1</v>
@@ -26147,10 +26147,10 @@
         <v>3</v>
       </c>
       <c r="IW51">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="IX51">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="IY51">
         <v>1</v>
@@ -26165,10 +26165,10 @@
         <v>1</v>
       </c>
       <c r="JC51">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="JD51">
-        <v>1</v>
+        <v>2</v>
       </c>
     </row>
     <row r="52" spans="1:264">
@@ -26647,28 +26647,28 @@
         <v>3</v>
       </c>
       <c r="IW52">
-        <v>4</v>
+        <v>1</v>
       </c>
       <c r="IX52">
+        <v>1</v>
+      </c>
+      <c r="IY52">
+        <v>1</v>
+      </c>
+      <c r="IZ52">
+        <v>1</v>
+      </c>
+      <c r="JA52">
+        <v>1</v>
+      </c>
+      <c r="JB52">
+        <v>1</v>
+      </c>
+      <c r="JC52">
+        <v>4</v>
+      </c>
+      <c r="JD52">
         <v>7</v>
-      </c>
-      <c r="IY52">
-        <v>1</v>
-      </c>
-      <c r="IZ52">
-        <v>1</v>
-      </c>
-      <c r="JA52">
-        <v>1</v>
-      </c>
-      <c r="JB52">
-        <v>1</v>
-      </c>
-      <c r="JC52">
-        <v>1</v>
-      </c>
-      <c r="JD52">
-        <v>1</v>
       </c>
     </row>
     <row r="53" spans="1:264">
@@ -27102,19 +27102,19 @@
         <v>3</v>
       </c>
       <c r="IW53">
+        <v>1</v>
+      </c>
+      <c r="IY53">
+        <v>1</v>
+      </c>
+      <c r="JA53">
+        <v>1</v>
+      </c>
+      <c r="JB53">
+        <v>0</v>
+      </c>
+      <c r="JC53">
         <v>7</v>
-      </c>
-      <c r="IY53">
-        <v>1</v>
-      </c>
-      <c r="JA53">
-        <v>1</v>
-      </c>
-      <c r="JC53">
-        <v>1</v>
-      </c>
-      <c r="JD53">
-        <v>0</v>
       </c>
     </row>
     <row r="54" spans="1:264">
@@ -27548,7 +27548,7 @@
         <v>3</v>
       </c>
       <c r="IW54">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="IY54">
         <v>1</v>
@@ -27556,11 +27556,11 @@
       <c r="JA54">
         <v>1</v>
       </c>
+      <c r="JB54">
+        <v>0</v>
+      </c>
       <c r="JC54">
-        <v>1</v>
-      </c>
-      <c r="JD54">
-        <v>0</v>
+        <v>2</v>
       </c>
     </row>
     <row r="55" spans="1:264">
@@ -27994,7 +27994,7 @@
         <v>3</v>
       </c>
       <c r="IW55">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="IY55">
         <v>1</v>
@@ -28002,11 +28002,11 @@
       <c r="JA55">
         <v>1</v>
       </c>
+      <c r="JB55">
+        <v>0</v>
+      </c>
       <c r="JC55">
-        <v>1</v>
-      </c>
-      <c r="JD55">
-        <v>0</v>
+        <v>2</v>
       </c>
     </row>
     <row r="56" spans="1:264">
@@ -28485,10 +28485,10 @@
         <v>1</v>
       </c>
       <c r="IW56">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="IX56">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="IY56">
         <v>1</v>
@@ -28503,10 +28503,10 @@
         <v>1</v>
       </c>
       <c r="JC56">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="JD56">
-        <v>1</v>
+        <v>2</v>
       </c>
     </row>
     <row r="57" spans="1:264">
@@ -28961,19 +28961,19 @@
         <v>1</v>
       </c>
       <c r="IX57">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="IZ57">
         <v>1</v>
       </c>
+      <c r="JA57">
+        <v>0</v>
+      </c>
       <c r="JB57">
         <v>1</v>
       </c>
-      <c r="JC57">
-        <v>0</v>
-      </c>
       <c r="JD57">
-        <v>1</v>
+        <v>2</v>
       </c>
     </row>
     <row r="58" spans="1:264">
@@ -29452,10 +29452,10 @@
         <v>1</v>
       </c>
       <c r="IW58">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="IX58">
-        <v>3</v>
+        <v>1</v>
       </c>
       <c r="IY58">
         <v>1</v>
@@ -29470,10 +29470,10 @@
         <v>1</v>
       </c>
       <c r="JC58">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="JD58">
-        <v>1</v>
+        <v>3</v>
       </c>
     </row>
     <row r="59" spans="1:264">
@@ -30452,10 +30452,10 @@
         <v>5</v>
       </c>
       <c r="IW60">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="IX60">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="IY60">
         <v>1</v>
@@ -30470,10 +30470,10 @@
         <v>1</v>
       </c>
       <c r="JC60">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="JD60">
-        <v>1</v>
+        <v>2</v>
       </c>
     </row>
     <row r="61" spans="1:264">
@@ -30952,10 +30952,10 @@
         <v>5</v>
       </c>
       <c r="IW61">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="IX61">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="IY61">
         <v>1</v>
@@ -30970,10 +30970,10 @@
         <v>1</v>
       </c>
       <c r="JC61">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="JD61">
-        <v>1</v>
+        <v>2</v>
       </c>
     </row>
     <row r="62" spans="1:264">
@@ -31952,28 +31952,28 @@
         <v>4</v>
       </c>
       <c r="IW63">
+        <v>1</v>
+      </c>
+      <c r="IX63">
+        <v>1</v>
+      </c>
+      <c r="IY63">
+        <v>1</v>
+      </c>
+      <c r="IZ63">
+        <v>1</v>
+      </c>
+      <c r="JA63">
+        <v>1</v>
+      </c>
+      <c r="JB63">
+        <v>1</v>
+      </c>
+      <c r="JC63">
         <v>6</v>
       </c>
-      <c r="IX63">
+      <c r="JD63">
         <v>6</v>
-      </c>
-      <c r="IY63">
-        <v>1</v>
-      </c>
-      <c r="IZ63">
-        <v>1</v>
-      </c>
-      <c r="JA63">
-        <v>1</v>
-      </c>
-      <c r="JB63">
-        <v>1</v>
-      </c>
-      <c r="JC63">
-        <v>1</v>
-      </c>
-      <c r="JD63">
-        <v>1</v>
       </c>
     </row>
     <row r="64" spans="1:264">
@@ -32452,10 +32452,10 @@
         <v>4</v>
       </c>
       <c r="IW64">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="IX64">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="IY64">
         <v>1</v>
@@ -32470,10 +32470,10 @@
         <v>1</v>
       </c>
       <c r="JC64">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="JD64">
-        <v>1</v>
+        <v>2</v>
       </c>
     </row>
     <row r="65" spans="1:264">
@@ -32952,28 +32952,28 @@
         <v>1</v>
       </c>
       <c r="IW65">
-        <v>4</v>
+        <v>1</v>
       </c>
       <c r="IX65">
+        <v>1</v>
+      </c>
+      <c r="IY65">
+        <v>1</v>
+      </c>
+      <c r="IZ65">
+        <v>1</v>
+      </c>
+      <c r="JA65">
+        <v>1</v>
+      </c>
+      <c r="JB65">
+        <v>1</v>
+      </c>
+      <c r="JC65">
+        <v>4</v>
+      </c>
+      <c r="JD65">
         <v>7</v>
-      </c>
-      <c r="IY65">
-        <v>1</v>
-      </c>
-      <c r="IZ65">
-        <v>1</v>
-      </c>
-      <c r="JA65">
-        <v>1</v>
-      </c>
-      <c r="JB65">
-        <v>1</v>
-      </c>
-      <c r="JC65">
-        <v>1</v>
-      </c>
-      <c r="JD65">
-        <v>1</v>
       </c>
     </row>
     <row r="66" spans="1:264">
@@ -33452,10 +33452,10 @@
         <v>1</v>
       </c>
       <c r="IW66">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="IX66">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="IY66">
         <v>1</v>
@@ -33470,10 +33470,10 @@
         <v>1</v>
       </c>
       <c r="JC66">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="JD66">
-        <v>1</v>
+        <v>2</v>
       </c>
     </row>
     <row r="67" spans="1:264">
@@ -33952,25 +33952,25 @@
         <v>1</v>
       </c>
       <c r="IW67">
+        <v>1</v>
+      </c>
+      <c r="IX67">
+        <v>1</v>
+      </c>
+      <c r="IY67">
+        <v>1</v>
+      </c>
+      <c r="IZ67">
+        <v>1</v>
+      </c>
+      <c r="JA67">
+        <v>1</v>
+      </c>
+      <c r="JB67">
+        <v>1</v>
+      </c>
+      <c r="JC67">
         <v>5</v>
-      </c>
-      <c r="IX67">
-        <v>1</v>
-      </c>
-      <c r="IY67">
-        <v>1</v>
-      </c>
-      <c r="IZ67">
-        <v>1</v>
-      </c>
-      <c r="JA67">
-        <v>1</v>
-      </c>
-      <c r="JB67">
-        <v>1</v>
-      </c>
-      <c r="JC67">
-        <v>1</v>
       </c>
       <c r="JD67">
         <v>1</v>
@@ -34455,25 +34455,25 @@
         <v>1</v>
       </c>
       <c r="IX68">
+        <v>1</v>
+      </c>
+      <c r="IY68">
+        <v>1</v>
+      </c>
+      <c r="IZ68">
+        <v>1</v>
+      </c>
+      <c r="JA68">
+        <v>1</v>
+      </c>
+      <c r="JB68">
+        <v>1</v>
+      </c>
+      <c r="JC68">
+        <v>1</v>
+      </c>
+      <c r="JD68">
         <v>7</v>
-      </c>
-      <c r="IY68">
-        <v>1</v>
-      </c>
-      <c r="IZ68">
-        <v>1</v>
-      </c>
-      <c r="JA68">
-        <v>1</v>
-      </c>
-      <c r="JB68">
-        <v>1</v>
-      </c>
-      <c r="JC68">
-        <v>1</v>
-      </c>
-      <c r="JD68">
-        <v>1</v>
       </c>
     </row>
     <row r="69" spans="1:264">
@@ -34928,7 +34928,7 @@
         <v>2</v>
       </c>
       <c r="IW69">
-        <v>4</v>
+        <v>1</v>
       </c>
       <c r="IY69">
         <v>1</v>
@@ -34936,11 +34936,11 @@
       <c r="JA69">
         <v>1</v>
       </c>
+      <c r="JB69">
+        <v>0</v>
+      </c>
       <c r="JC69">
         <v>1</v>
-      </c>
-      <c r="JD69">
-        <v>0</v>
       </c>
     </row>
     <row r="70" spans="1:264">
@@ -35419,10 +35419,10 @@
         <v>1</v>
       </c>
       <c r="IW70">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="IX70">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="IY70">
         <v>1</v>
@@ -35437,10 +35437,10 @@
         <v>1</v>
       </c>
       <c r="JC70">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="JD70">
-        <v>1</v>
+        <v>2</v>
       </c>
     </row>
     <row r="71" spans="1:264">
@@ -35919,28 +35919,28 @@
         <v>1</v>
       </c>
       <c r="IW71">
+        <v>1</v>
+      </c>
+      <c r="IX71">
+        <v>1</v>
+      </c>
+      <c r="IY71">
+        <v>1</v>
+      </c>
+      <c r="IZ71">
+        <v>1</v>
+      </c>
+      <c r="JA71">
+        <v>1</v>
+      </c>
+      <c r="JB71">
+        <v>1</v>
+      </c>
+      <c r="JC71">
         <v>7</v>
       </c>
-      <c r="IX71">
-        <v>2</v>
-      </c>
-      <c r="IY71">
-        <v>1</v>
-      </c>
-      <c r="IZ71">
-        <v>1</v>
-      </c>
-      <c r="JA71">
-        <v>1</v>
-      </c>
-      <c r="JB71">
-        <v>1</v>
-      </c>
-      <c r="JC71">
-        <v>1</v>
-      </c>
       <c r="JD71">
-        <v>1</v>
+        <v>2</v>
       </c>
     </row>
     <row r="72" spans="1:264">
@@ -36900,26 +36900,26 @@
       <c r="IV73">
         <v>1</v>
       </c>
-      <c r="IW73">
-        <v>2</v>
-      </c>
       <c r="IX73">
-        <v>2</v>
+        <v>1</v>
+      </c>
+      <c r="IY73">
+        <v>1</v>
       </c>
       <c r="IZ73">
         <v>1</v>
       </c>
       <c r="JA73">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="JB73">
         <v>1</v>
       </c>
       <c r="JC73">
-        <v>0</v>
+        <v>2</v>
       </c>
       <c r="JD73">
-        <v>1</v>
+        <v>2</v>
       </c>
     </row>
     <row r="74" spans="1:264">
@@ -37313,10 +37313,10 @@
       <c r="IN74">
         <v>2</v>
       </c>
-      <c r="JC74">
-        <v>0</v>
-      </c>
-      <c r="JD74">
+      <c r="JA74">
+        <v>0</v>
+      </c>
+      <c r="JB74">
         <v>0</v>
       </c>
     </row>
@@ -37711,10 +37711,10 @@
       <c r="IN75">
         <v>2</v>
       </c>
-      <c r="JC75">
-        <v>0</v>
-      </c>
-      <c r="JD75">
+      <c r="JA75">
+        <v>0</v>
+      </c>
+      <c r="JB75">
         <v>0</v>
       </c>
     </row>
@@ -38109,10 +38109,10 @@
       <c r="IN76">
         <v>2</v>
       </c>
-      <c r="JC76">
-        <v>0</v>
-      </c>
-      <c r="JD76">
+      <c r="JA76">
+        <v>0</v>
+      </c>
+      <c r="JB76">
         <v>0</v>
       </c>
     </row>
@@ -39095,7 +39095,7 @@
         <v>1</v>
       </c>
       <c r="IX78">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="IY78">
         <v>1</v>
@@ -39113,7 +39113,7 @@
         <v>1</v>
       </c>
       <c r="JD78">
-        <v>1</v>
+        <v>2</v>
       </c>
     </row>
     <row r="79" spans="1:264">
@@ -39592,10 +39592,10 @@
         <v>3</v>
       </c>
       <c r="IW79">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="IX79">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="IY79">
         <v>1</v>
@@ -39610,10 +39610,10 @@
         <v>1</v>
       </c>
       <c r="JC79">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="JD79">
-        <v>1</v>
+        <v>2</v>
       </c>
     </row>
     <row r="80" spans="1:264">
@@ -40092,28 +40092,28 @@
         <v>3</v>
       </c>
       <c r="IW80">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="IX80">
+        <v>1</v>
+      </c>
+      <c r="IY80">
+        <v>1</v>
+      </c>
+      <c r="IZ80">
+        <v>1</v>
+      </c>
+      <c r="JA80">
+        <v>1</v>
+      </c>
+      <c r="JB80">
+        <v>1</v>
+      </c>
+      <c r="JC80">
+        <v>2</v>
+      </c>
+      <c r="JD80">
         <v>7</v>
-      </c>
-      <c r="IY80">
-        <v>1</v>
-      </c>
-      <c r="IZ80">
-        <v>1</v>
-      </c>
-      <c r="JA80">
-        <v>1</v>
-      </c>
-      <c r="JB80">
-        <v>1</v>
-      </c>
-      <c r="JC80">
-        <v>1</v>
-      </c>
-      <c r="JD80">
-        <v>1</v>
       </c>
     </row>
     <row r="81" spans="1:264">
@@ -40592,28 +40592,28 @@
         <v>3</v>
       </c>
       <c r="IW81">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="IX81">
+        <v>1</v>
+      </c>
+      <c r="IY81">
+        <v>1</v>
+      </c>
+      <c r="IZ81">
+        <v>1</v>
+      </c>
+      <c r="JA81">
+        <v>1</v>
+      </c>
+      <c r="JB81">
+        <v>1</v>
+      </c>
+      <c r="JC81">
+        <v>2</v>
+      </c>
+      <c r="JD81">
         <v>6</v>
-      </c>
-      <c r="IY81">
-        <v>1</v>
-      </c>
-      <c r="IZ81">
-        <v>1</v>
-      </c>
-      <c r="JA81">
-        <v>1</v>
-      </c>
-      <c r="JB81">
-        <v>1</v>
-      </c>
-      <c r="JC81">
-        <v>1</v>
-      </c>
-      <c r="JD81">
-        <v>1</v>
       </c>
     </row>
     <row r="82" spans="1:264">
@@ -41092,10 +41092,10 @@
         <v>3</v>
       </c>
       <c r="IW82">
-        <v>4</v>
+        <v>1</v>
       </c>
       <c r="IX82">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="IY82">
         <v>1</v>
@@ -41110,10 +41110,10 @@
         <v>1</v>
       </c>
       <c r="JC82">
-        <v>1</v>
+        <v>4</v>
       </c>
       <c r="JD82">
-        <v>1</v>
+        <v>2</v>
       </c>
     </row>
     <row r="83" spans="1:264">
@@ -41507,10 +41507,10 @@
       <c r="IN83">
         <v>3</v>
       </c>
-      <c r="JC83">
-        <v>0</v>
-      </c>
-      <c r="JD83">
+      <c r="JA83">
+        <v>0</v>
+      </c>
+      <c r="JB83">
         <v>0</v>
       </c>
     </row>
@@ -41905,10 +41905,10 @@
       <c r="IN84">
         <v>2</v>
       </c>
-      <c r="JC84">
-        <v>0</v>
-      </c>
-      <c r="JD84">
+      <c r="JA84">
+        <v>0</v>
+      </c>
+      <c r="JB84">
         <v>0</v>
       </c>
     </row>
@@ -42303,10 +42303,10 @@
       <c r="IN85">
         <v>2</v>
       </c>
-      <c r="JC85">
-        <v>0</v>
-      </c>
-      <c r="JD85">
+      <c r="JA85">
+        <v>0</v>
+      </c>
+      <c r="JB85">
         <v>0</v>
       </c>
     </row>
@@ -42741,7 +42741,7 @@
         <v>5</v>
       </c>
       <c r="IW86">
-        <v>3</v>
+        <v>1</v>
       </c>
       <c r="IY86">
         <v>1</v>
@@ -42749,11 +42749,11 @@
       <c r="JA86">
         <v>1</v>
       </c>
+      <c r="JB86">
+        <v>0</v>
+      </c>
       <c r="JC86">
-        <v>1</v>
-      </c>
-      <c r="JD86">
-        <v>0</v>
+        <v>3</v>
       </c>
     </row>
     <row r="87" spans="1:264">
@@ -43187,19 +43187,19 @@
         <v>5</v>
       </c>
       <c r="IW87">
+        <v>1</v>
+      </c>
+      <c r="IY87">
+        <v>1</v>
+      </c>
+      <c r="JA87">
+        <v>1</v>
+      </c>
+      <c r="JB87">
+        <v>0</v>
+      </c>
+      <c r="JC87">
         <v>7</v>
-      </c>
-      <c r="IY87">
-        <v>1</v>
-      </c>
-      <c r="JA87">
-        <v>1</v>
-      </c>
-      <c r="JC87">
-        <v>1</v>
-      </c>
-      <c r="JD87">
-        <v>0</v>
       </c>
     </row>
     <row r="88" spans="1:264">
@@ -43608,10 +43608,10 @@
       <c r="IN88">
         <v>3</v>
       </c>
-      <c r="JC88">
-        <v>0</v>
-      </c>
-      <c r="JD88">
+      <c r="JA88">
+        <v>0</v>
+      </c>
+      <c r="JB88">
         <v>0</v>
       </c>
     </row>
@@ -44094,25 +44094,25 @@
         <v>1</v>
       </c>
       <c r="IX89">
+        <v>1</v>
+      </c>
+      <c r="IY89">
+        <v>1</v>
+      </c>
+      <c r="IZ89">
+        <v>1</v>
+      </c>
+      <c r="JA89">
+        <v>1</v>
+      </c>
+      <c r="JB89">
+        <v>1</v>
+      </c>
+      <c r="JC89">
+        <v>1</v>
+      </c>
+      <c r="JD89">
         <v>7</v>
-      </c>
-      <c r="IY89">
-        <v>1</v>
-      </c>
-      <c r="IZ89">
-        <v>1</v>
-      </c>
-      <c r="JA89">
-        <v>1</v>
-      </c>
-      <c r="JB89">
-        <v>1</v>
-      </c>
-      <c r="JC89">
-        <v>1</v>
-      </c>
-      <c r="JD89">
-        <v>1</v>
       </c>
     </row>
     <row r="90" spans="1:264">
@@ -44594,7 +44594,7 @@
         <v>1</v>
       </c>
       <c r="IX90">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="IY90">
         <v>1</v>
@@ -44612,7 +44612,7 @@
         <v>1</v>
       </c>
       <c r="JD90">
-        <v>1</v>
+        <v>2</v>
       </c>
     </row>
     <row r="91" spans="1:264">
@@ -45091,7 +45091,7 @@
         <v>5</v>
       </c>
       <c r="IW91">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="IX91">
         <v>1</v>
@@ -45109,7 +45109,7 @@
         <v>1</v>
       </c>
       <c r="JC91">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="JD91">
         <v>1</v>
@@ -46097,10 +46097,10 @@
         <v>2</v>
       </c>
       <c r="IW93">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="IX93">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="IY93">
         <v>1</v>
@@ -46115,10 +46115,10 @@
         <v>1</v>
       </c>
       <c r="JC93">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="JD93">
-        <v>1</v>
+        <v>2</v>
       </c>
     </row>
     <row r="94" spans="1:264">
@@ -46600,7 +46600,7 @@
         <v>2</v>
       </c>
       <c r="IW94">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="IX94">
         <v>1</v>
@@ -46618,7 +46618,7 @@
         <v>1</v>
       </c>
       <c r="JC94">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="JD94">
         <v>1</v>
@@ -47103,10 +47103,10 @@
         <v>1</v>
       </c>
       <c r="IW95">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="IX95">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="IY95">
         <v>1</v>
@@ -47121,10 +47121,10 @@
         <v>1</v>
       </c>
       <c r="JC95">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="JD95">
-        <v>1</v>
+        <v>2</v>
       </c>
     </row>
     <row r="96" spans="1:264">
@@ -47606,7 +47606,7 @@
         <v>1</v>
       </c>
       <c r="IW96">
-        <v>4</v>
+        <v>1</v>
       </c>
       <c r="IX96">
         <v>1</v>
@@ -47624,7 +47624,7 @@
         <v>1</v>
       </c>
       <c r="JC96">
-        <v>1</v>
+        <v>4</v>
       </c>
       <c r="JD96">
         <v>1</v>
@@ -48109,10 +48109,10 @@
         <v>1</v>
       </c>
       <c r="IW97">
-        <v>4</v>
+        <v>1</v>
       </c>
       <c r="IX97">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="IY97">
         <v>1</v>
@@ -48127,10 +48127,10 @@
         <v>1</v>
       </c>
       <c r="JC97">
-        <v>1</v>
+        <v>4</v>
       </c>
       <c r="JD97">
-        <v>1</v>
+        <v>2</v>
       </c>
     </row>
     <row r="98" spans="1:264">
@@ -48567,7 +48567,7 @@
         <v>1</v>
       </c>
       <c r="IW98">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="IY98">
         <v>1</v>
@@ -48575,11 +48575,11 @@
       <c r="JA98">
         <v>1</v>
       </c>
+      <c r="JB98">
+        <v>0</v>
+      </c>
       <c r="JC98">
-        <v>1</v>
-      </c>
-      <c r="JD98">
-        <v>0</v>
+        <v>2</v>
       </c>
     </row>
     <row r="99" spans="1:264">
@@ -49016,19 +49016,19 @@
         <v>1</v>
       </c>
       <c r="IW99">
+        <v>1</v>
+      </c>
+      <c r="IY99">
+        <v>1</v>
+      </c>
+      <c r="JA99">
+        <v>1</v>
+      </c>
+      <c r="JB99">
+        <v>0</v>
+      </c>
+      <c r="JC99">
         <v>6</v>
-      </c>
-      <c r="IY99">
-        <v>1</v>
-      </c>
-      <c r="JA99">
-        <v>1</v>
-      </c>
-      <c r="JC99">
-        <v>1</v>
-      </c>
-      <c r="JD99">
-        <v>0</v>
       </c>
     </row>
     <row r="100" spans="1:264">
@@ -49465,7 +49465,7 @@
         <v>1</v>
       </c>
       <c r="IW100">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="IY100">
         <v>1</v>
@@ -49473,11 +49473,11 @@
       <c r="JA100">
         <v>1</v>
       </c>
+      <c r="JB100">
+        <v>0</v>
+      </c>
       <c r="JC100">
-        <v>1</v>
-      </c>
-      <c r="JD100">
-        <v>0</v>
+        <v>2</v>
       </c>
     </row>
     <row r="101" spans="1:264">
@@ -49959,10 +49959,10 @@
         <v>4</v>
       </c>
       <c r="IW101">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="IX101">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="IY101">
         <v>1</v>
@@ -49977,10 +49977,10 @@
         <v>1</v>
       </c>
       <c r="JC101">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="JD101">
-        <v>1</v>
+        <v>2</v>
       </c>
     </row>
     <row r="102" spans="1:264">
@@ -50462,10 +50462,10 @@
         <v>4</v>
       </c>
       <c r="IW102">
-        <v>4</v>
+        <v>1</v>
       </c>
       <c r="IX102">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="IY102">
         <v>1</v>
@@ -50480,10 +50480,10 @@
         <v>1</v>
       </c>
       <c r="JC102">
-        <v>1</v>
+        <v>4</v>
       </c>
       <c r="JD102">
-        <v>1</v>
+        <v>2</v>
       </c>
     </row>
     <row r="103" spans="1:264">
@@ -50965,7 +50965,7 @@
         <v>4</v>
       </c>
       <c r="IW103">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="IX103">
         <v>1</v>
@@ -50983,7 +50983,7 @@
         <v>1</v>
       </c>
       <c r="JC103">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="JD103">
         <v>1</v>
@@ -51468,7 +51468,7 @@
         <v>1</v>
       </c>
       <c r="IW104">
-        <v>3</v>
+        <v>1</v>
       </c>
       <c r="IX104">
         <v>1</v>
@@ -51486,7 +51486,7 @@
         <v>1</v>
       </c>
       <c r="JC104">
-        <v>1</v>
+        <v>3</v>
       </c>
       <c r="JD104">
         <v>1</v>
@@ -51971,10 +51971,10 @@
         <v>1</v>
       </c>
       <c r="IW105">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="IX105">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="IY105">
         <v>1</v>
@@ -51989,10 +51989,10 @@
         <v>1</v>
       </c>
       <c r="JC105">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="JD105">
-        <v>1</v>
+        <v>2</v>
       </c>
     </row>
     <row r="106" spans="1:264">
@@ -52474,10 +52474,10 @@
         <v>1</v>
       </c>
       <c r="IW106">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="IX106">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="IY106">
         <v>1</v>
@@ -52492,10 +52492,10 @@
         <v>1</v>
       </c>
       <c r="JC106">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="JD106">
-        <v>1</v>
+        <v>2</v>
       </c>
     </row>
     <row r="107" spans="1:264">
@@ -52977,10 +52977,10 @@
         <v>5</v>
       </c>
       <c r="IW107">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="IX107">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="IY107">
         <v>1</v>
@@ -52995,10 +52995,10 @@
         <v>1</v>
       </c>
       <c r="JC107">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="JD107">
-        <v>1</v>
+        <v>2</v>
       </c>
     </row>
     <row r="108" spans="1:264">
@@ -53480,10 +53480,10 @@
         <v>5</v>
       </c>
       <c r="IW108">
-        <v>4</v>
+        <v>1</v>
       </c>
       <c r="IX108">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="IY108">
         <v>1</v>
@@ -53498,10 +53498,10 @@
         <v>1</v>
       </c>
       <c r="JC108">
-        <v>1</v>
+        <v>4</v>
       </c>
       <c r="JD108">
-        <v>1</v>
+        <v>2</v>
       </c>
     </row>
     <row r="109" spans="1:264">
@@ -53983,10 +53983,10 @@
         <v>5</v>
       </c>
       <c r="IW109">
-        <v>4</v>
+        <v>1</v>
       </c>
       <c r="IX109">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="IY109">
         <v>1</v>
@@ -54001,10 +54001,10 @@
         <v>1</v>
       </c>
       <c r="JC109">
-        <v>1</v>
+        <v>4</v>
       </c>
       <c r="JD109">
-        <v>1</v>
+        <v>2</v>
       </c>
     </row>
     <row r="110" spans="1:264">
@@ -54486,10 +54486,10 @@
         <v>4</v>
       </c>
       <c r="IW110">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="IX110">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="IY110">
         <v>1</v>
@@ -54504,10 +54504,10 @@
         <v>1</v>
       </c>
       <c r="JC110">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="JD110">
-        <v>1</v>
+        <v>2</v>
       </c>
     </row>
     <row r="111" spans="1:264">
@@ -54989,10 +54989,10 @@
         <v>4</v>
       </c>
       <c r="IW111">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="IX111">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="IY111">
         <v>1</v>
@@ -55007,10 +55007,10 @@
         <v>1</v>
       </c>
       <c r="JC111">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="JD111">
-        <v>1</v>
+        <v>2</v>
       </c>
     </row>
     <row r="112" spans="1:264">
@@ -55492,7 +55492,7 @@
         <v>4</v>
       </c>
       <c r="IW112">
-        <v>3</v>
+        <v>1</v>
       </c>
       <c r="IX112">
         <v>1</v>
@@ -55510,7 +55510,7 @@
         <v>1</v>
       </c>
       <c r="JC112">
-        <v>1</v>
+        <v>3</v>
       </c>
       <c r="JD112">
         <v>1</v>
@@ -55910,10 +55910,10 @@
       <c r="IN113">
         <v>2</v>
       </c>
-      <c r="JC113">
-        <v>0</v>
-      </c>
-      <c r="JD113">
+      <c r="JA113">
+        <v>0</v>
+      </c>
+      <c r="JB113">
         <v>0</v>
       </c>
     </row>
@@ -56311,10 +56311,10 @@
       <c r="IN114">
         <v>2</v>
       </c>
-      <c r="JC114">
-        <v>0</v>
-      </c>
-      <c r="JD114">
+      <c r="JA114">
+        <v>0</v>
+      </c>
+      <c r="JB114">
         <v>0</v>
       </c>
     </row>
@@ -56712,10 +56712,10 @@
       <c r="IN115">
         <v>2</v>
       </c>
-      <c r="JC115">
-        <v>0</v>
-      </c>
-      <c r="JD115">
+      <c r="JA115">
+        <v>0</v>
+      </c>
+      <c r="JB115">
         <v>0</v>
       </c>
     </row>
@@ -57198,10 +57198,10 @@
         <v>1</v>
       </c>
       <c r="IW116">
-        <v>3</v>
+        <v>1</v>
       </c>
       <c r="IX116">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="IY116">
         <v>1</v>
@@ -57216,10 +57216,10 @@
         <v>1</v>
       </c>
       <c r="JC116">
-        <v>1</v>
+        <v>3</v>
       </c>
       <c r="JD116">
-        <v>1</v>
+        <v>2</v>
       </c>
     </row>
     <row r="117" spans="1:264">
@@ -57701,7 +57701,7 @@
         <v>1</v>
       </c>
       <c r="IW117">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="IX117">
         <v>1</v>
@@ -57719,7 +57719,7 @@
         <v>1</v>
       </c>
       <c r="JC117">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="JD117">
         <v>1</v>
@@ -58204,10 +58204,10 @@
         <v>1</v>
       </c>
       <c r="IW118">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="IX118">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="IY118">
         <v>1</v>
@@ -58222,10 +58222,10 @@
         <v>1</v>
       </c>
       <c r="JC118">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="JD118">
-        <v>1</v>
+        <v>2</v>
       </c>
     </row>
     <row r="119" spans="1:264">
@@ -58707,7 +58707,7 @@
         <v>4</v>
       </c>
       <c r="IW119">
-        <v>3</v>
+        <v>1</v>
       </c>
       <c r="IX119">
         <v>1</v>
@@ -58725,10 +58725,10 @@
         <v>1</v>
       </c>
       <c r="JC119">
-        <v>1</v>
+        <v>3</v>
       </c>
       <c r="JD119">
-        <v>1</v>
+        <v>3</v>
       </c>
     </row>
     <row r="120" spans="1:264">
@@ -59210,10 +59210,10 @@
         <v>4</v>
       </c>
       <c r="IW120">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="IX120">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="IY120">
         <v>1</v>
@@ -59228,10 +59228,10 @@
         <v>1</v>
       </c>
       <c r="JC120">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="JD120">
-        <v>1</v>
+        <v>2</v>
       </c>
     </row>
     <row r="121" spans="1:264">
@@ -59713,28 +59713,28 @@
         <v>4</v>
       </c>
       <c r="IW121">
+        <v>1</v>
+      </c>
+      <c r="IX121">
+        <v>1</v>
+      </c>
+      <c r="IY121">
+        <v>0</v>
+      </c>
+      <c r="IZ121">
+        <v>0</v>
+      </c>
+      <c r="JA121">
+        <v>1</v>
+      </c>
+      <c r="JB121">
+        <v>1</v>
+      </c>
+      <c r="JC121">
         <v>5</v>
       </c>
-      <c r="IX121">
+      <c r="JD121">
         <v>5</v>
-      </c>
-      <c r="IY121">
-        <v>1</v>
-      </c>
-      <c r="IZ121">
-        <v>1</v>
-      </c>
-      <c r="JA121">
-        <v>0</v>
-      </c>
-      <c r="JB121">
-        <v>0</v>
-      </c>
-      <c r="JC121">
-        <v>1</v>
-      </c>
-      <c r="JD121">
-        <v>1</v>
       </c>
     </row>
     <row r="122" spans="1:264">
@@ -60171,7 +60171,7 @@
         <v>3</v>
       </c>
       <c r="IW122">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="IY122">
         <v>1</v>
@@ -60179,11 +60179,11 @@
       <c r="JA122">
         <v>1</v>
       </c>
+      <c r="JB122">
+        <v>0</v>
+      </c>
       <c r="JC122">
-        <v>1</v>
-      </c>
-      <c r="JD122">
-        <v>0</v>
+        <v>2</v>
       </c>
     </row>
     <row r="123" spans="1:264">
@@ -60620,7 +60620,7 @@
         <v>3</v>
       </c>
       <c r="IW123">
-        <v>4</v>
+        <v>1</v>
       </c>
       <c r="IY123">
         <v>1</v>
@@ -60628,11 +60628,11 @@
       <c r="JA123">
         <v>1</v>
       </c>
+      <c r="JB123">
+        <v>0</v>
+      </c>
       <c r="JC123">
-        <v>1</v>
-      </c>
-      <c r="JD123">
-        <v>0</v>
+        <v>4</v>
       </c>
     </row>
     <row r="124" spans="1:264">
@@ -61069,7 +61069,7 @@
         <v>3</v>
       </c>
       <c r="IW124">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="IY124">
         <v>1</v>
@@ -61077,11 +61077,11 @@
       <c r="JA124">
         <v>1</v>
       </c>
+      <c r="JB124">
+        <v>0</v>
+      </c>
       <c r="JC124">
-        <v>1</v>
-      </c>
-      <c r="JD124">
-        <v>0</v>
+        <v>2</v>
       </c>
     </row>
     <row r="125" spans="1:264">
@@ -61563,28 +61563,28 @@
         <v>3</v>
       </c>
       <c r="IW125">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="IX125">
+        <v>1</v>
+      </c>
+      <c r="IY125">
+        <v>1</v>
+      </c>
+      <c r="IZ125">
+        <v>1</v>
+      </c>
+      <c r="JA125">
+        <v>1</v>
+      </c>
+      <c r="JB125">
+        <v>1</v>
+      </c>
+      <c r="JC125">
+        <v>2</v>
+      </c>
+      <c r="JD125">
         <v>7</v>
-      </c>
-      <c r="IY125">
-        <v>1</v>
-      </c>
-      <c r="IZ125">
-        <v>1</v>
-      </c>
-      <c r="JA125">
-        <v>1</v>
-      </c>
-      <c r="JB125">
-        <v>1</v>
-      </c>
-      <c r="JC125">
-        <v>1</v>
-      </c>
-      <c r="JD125">
-        <v>1</v>
       </c>
     </row>
     <row r="126" spans="1:264">
@@ -62066,7 +62066,7 @@
         <v>3</v>
       </c>
       <c r="IW126">
-        <v>4</v>
+        <v>1</v>
       </c>
       <c r="IX126">
         <v>1</v>
@@ -62084,7 +62084,7 @@
         <v>1</v>
       </c>
       <c r="JC126">
-        <v>1</v>
+        <v>4</v>
       </c>
       <c r="JD126">
         <v>1</v>
@@ -62572,7 +62572,7 @@
         <v>1</v>
       </c>
       <c r="IX127">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="IY127">
         <v>1</v>
@@ -62590,7 +62590,7 @@
         <v>1</v>
       </c>
       <c r="JD127">
-        <v>1</v>
+        <v>2</v>
       </c>
     </row>
     <row r="128" spans="1:264">
@@ -63048,7 +63048,7 @@
         <v>3</v>
       </c>
       <c r="IW128">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="IY128">
         <v>1</v>
@@ -63056,11 +63056,11 @@
       <c r="JA128">
         <v>1</v>
       </c>
+      <c r="JB128">
+        <v>0</v>
+      </c>
       <c r="JC128">
-        <v>1</v>
-      </c>
-      <c r="JD128">
-        <v>0</v>
+        <v>2</v>
       </c>
     </row>
     <row r="129" spans="1:264">
@@ -63542,10 +63542,10 @@
         <v>1</v>
       </c>
       <c r="IW129">
-        <v>4</v>
+        <v>1</v>
       </c>
       <c r="IX129">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="IY129">
         <v>1</v>
@@ -63560,10 +63560,10 @@
         <v>1</v>
       </c>
       <c r="JC129">
-        <v>1</v>
+        <v>4</v>
       </c>
       <c r="JD129">
-        <v>1</v>
+        <v>2</v>
       </c>
     </row>
     <row r="130" spans="1:264">
@@ -64045,10 +64045,10 @@
         <v>1</v>
       </c>
       <c r="IW130">
-        <v>3</v>
+        <v>1</v>
       </c>
       <c r="IX130">
-        <v>3</v>
+        <v>1</v>
       </c>
       <c r="IY130">
         <v>1</v>
@@ -64063,10 +64063,10 @@
         <v>1</v>
       </c>
       <c r="JC130">
-        <v>1</v>
+        <v>3</v>
       </c>
       <c r="JD130">
-        <v>1</v>
+        <v>3</v>
       </c>
     </row>
     <row r="131" spans="1:264">
@@ -64509,7 +64509,7 @@
         <v>1</v>
       </c>
       <c r="IW131">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="IY131">
         <v>1</v>
@@ -64517,11 +64517,11 @@
       <c r="JA131">
         <v>1</v>
       </c>
+      <c r="JB131">
+        <v>0</v>
+      </c>
       <c r="JC131">
-        <v>1</v>
-      </c>
-      <c r="JD131">
-        <v>0</v>
+        <v>2</v>
       </c>
     </row>
     <row r="132" spans="1:264">
@@ -64964,7 +64964,7 @@
         <v>1</v>
       </c>
       <c r="IW132">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="IY132">
         <v>1</v>
@@ -64972,11 +64972,11 @@
       <c r="JA132">
         <v>1</v>
       </c>
+      <c r="JB132">
+        <v>0</v>
+      </c>
       <c r="JC132">
-        <v>1</v>
-      </c>
-      <c r="JD132">
-        <v>0</v>
+        <v>2</v>
       </c>
     </row>
     <row r="133" spans="1:264">
@@ -65419,19 +65419,19 @@
         <v>1</v>
       </c>
       <c r="IW133">
+        <v>1</v>
+      </c>
+      <c r="IY133">
+        <v>1</v>
+      </c>
+      <c r="JA133">
+        <v>1</v>
+      </c>
+      <c r="JB133">
+        <v>0</v>
+      </c>
+      <c r="JC133">
         <v>7</v>
-      </c>
-      <c r="IY133">
-        <v>1</v>
-      </c>
-      <c r="JA133">
-        <v>1</v>
-      </c>
-      <c r="JC133">
-        <v>1</v>
-      </c>
-      <c r="JD133">
-        <v>0</v>
       </c>
     </row>
     <row r="134" spans="1:264">
@@ -65874,19 +65874,19 @@
         <v>5</v>
       </c>
       <c r="IX134">
-        <v>4</v>
+        <v>1</v>
       </c>
       <c r="IZ134">
         <v>1</v>
       </c>
+      <c r="JA134">
+        <v>0</v>
+      </c>
       <c r="JB134">
         <v>1</v>
       </c>
-      <c r="JC134">
-        <v>0</v>
-      </c>
       <c r="JD134">
-        <v>1</v>
+        <v>7</v>
       </c>
     </row>
     <row r="135" spans="1:264">
@@ -66329,19 +66329,19 @@
         <v>5</v>
       </c>
       <c r="IX135">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="IZ135">
         <v>1</v>
       </c>
+      <c r="JA135">
+        <v>0</v>
+      </c>
       <c r="JB135">
         <v>1</v>
       </c>
-      <c r="JC135">
-        <v>0</v>
-      </c>
       <c r="JD135">
-        <v>1</v>
+        <v>2</v>
       </c>
     </row>
     <row r="136" spans="1:264">
@@ -66784,19 +66784,19 @@
         <v>5</v>
       </c>
       <c r="IX136">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="IZ136">
         <v>1</v>
       </c>
+      <c r="JA136">
+        <v>0</v>
+      </c>
       <c r="JB136">
         <v>1</v>
       </c>
-      <c r="JC136">
-        <v>0</v>
-      </c>
       <c r="JD136">
-        <v>1</v>
+        <v>2</v>
       </c>
     </row>
     <row r="137" spans="1:264">
@@ -67193,10 +67193,10 @@
       <c r="IN137">
         <v>3</v>
       </c>
-      <c r="JC137">
-        <v>0</v>
-      </c>
-      <c r="JD137">
+      <c r="JA137">
+        <v>0</v>
+      </c>
+      <c r="JB137">
         <v>0</v>
       </c>
     </row>
@@ -67594,10 +67594,10 @@
       <c r="IN138">
         <v>2</v>
       </c>
-      <c r="JC138">
-        <v>0</v>
-      </c>
-      <c r="JD138">
+      <c r="JA138">
+        <v>0</v>
+      </c>
+      <c r="JB138">
         <v>0</v>
       </c>
     </row>
@@ -67995,10 +67995,10 @@
       <c r="IN139">
         <v>2</v>
       </c>
-      <c r="JC139">
-        <v>0</v>
-      </c>
-      <c r="JD139">
+      <c r="JA139">
+        <v>0</v>
+      </c>
+      <c r="JB139">
         <v>0</v>
       </c>
     </row>
@@ -68478,10 +68478,10 @@
         <v>3</v>
       </c>
       <c r="IW140">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="IX140">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="IY140">
         <v>1</v>
@@ -68496,10 +68496,10 @@
         <v>1</v>
       </c>
       <c r="JC140">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="JD140">
-        <v>1</v>
+        <v>2</v>
       </c>
     </row>
     <row r="141" spans="1:264">
@@ -68978,7 +68978,7 @@
         <v>3</v>
       </c>
       <c r="IW141">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="IX141">
         <v>1</v>
@@ -68996,7 +68996,7 @@
         <v>1</v>
       </c>
       <c r="JC141">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="JD141">
         <v>1</v>
@@ -69478,28 +69478,28 @@
         <v>3</v>
       </c>
       <c r="IW142">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="IX142">
+        <v>1</v>
+      </c>
+      <c r="IY142">
+        <v>1</v>
+      </c>
+      <c r="IZ142">
+        <v>1</v>
+      </c>
+      <c r="JA142">
+        <v>1</v>
+      </c>
+      <c r="JB142">
+        <v>1</v>
+      </c>
+      <c r="JC142">
+        <v>2</v>
+      </c>
+      <c r="JD142">
         <v>7</v>
-      </c>
-      <c r="IY142">
-        <v>1</v>
-      </c>
-      <c r="IZ142">
-        <v>1</v>
-      </c>
-      <c r="JA142">
-        <v>1</v>
-      </c>
-      <c r="JB142">
-        <v>1</v>
-      </c>
-      <c r="JC142">
-        <v>1</v>
-      </c>
-      <c r="JD142">
-        <v>1</v>
       </c>
     </row>
     <row r="143" spans="1:264">
@@ -69978,28 +69978,28 @@
         <v>5</v>
       </c>
       <c r="IW143">
-        <v>4</v>
+        <v>1</v>
       </c>
       <c r="IX143">
+        <v>1</v>
+      </c>
+      <c r="IY143">
+        <v>1</v>
+      </c>
+      <c r="IZ143">
+        <v>1</v>
+      </c>
+      <c r="JA143">
+        <v>1</v>
+      </c>
+      <c r="JB143">
+        <v>1</v>
+      </c>
+      <c r="JC143">
+        <v>4</v>
+      </c>
+      <c r="JD143">
         <v>5</v>
-      </c>
-      <c r="IY143">
-        <v>1</v>
-      </c>
-      <c r="IZ143">
-        <v>1</v>
-      </c>
-      <c r="JA143">
-        <v>1</v>
-      </c>
-      <c r="JB143">
-        <v>1</v>
-      </c>
-      <c r="JC143">
-        <v>1</v>
-      </c>
-      <c r="JD143">
-        <v>1</v>
       </c>
     </row>
     <row r="144" spans="1:264">
@@ -70481,25 +70481,25 @@
         <v>1</v>
       </c>
       <c r="IX144">
+        <v>1</v>
+      </c>
+      <c r="IY144">
+        <v>1</v>
+      </c>
+      <c r="IZ144">
+        <v>1</v>
+      </c>
+      <c r="JA144">
+        <v>1</v>
+      </c>
+      <c r="JB144">
+        <v>1</v>
+      </c>
+      <c r="JC144">
+        <v>1</v>
+      </c>
+      <c r="JD144">
         <v>6</v>
-      </c>
-      <c r="IY144">
-        <v>1</v>
-      </c>
-      <c r="IZ144">
-        <v>1</v>
-      </c>
-      <c r="JA144">
-        <v>1</v>
-      </c>
-      <c r="JB144">
-        <v>1</v>
-      </c>
-      <c r="JC144">
-        <v>1</v>
-      </c>
-      <c r="JD144">
-        <v>1</v>
       </c>
     </row>
     <row r="145" spans="1:264">
@@ -70978,10 +70978,10 @@
         <v>5</v>
       </c>
       <c r="IW145">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="IX145">
-        <v>4</v>
+        <v>1</v>
       </c>
       <c r="IY145">
         <v>1</v>
@@ -70996,10 +70996,10 @@
         <v>1</v>
       </c>
       <c r="JC145">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="JD145">
-        <v>1</v>
+        <v>7</v>
       </c>
     </row>
     <row r="146" spans="1:264">
@@ -71478,10 +71478,10 @@
         <v>5</v>
       </c>
       <c r="IW146">
-        <v>3</v>
+        <v>1</v>
       </c>
       <c r="IX146">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="IY146">
         <v>1</v>
@@ -71496,10 +71496,10 @@
         <v>1</v>
       </c>
       <c r="JC146">
-        <v>1</v>
+        <v>3</v>
       </c>
       <c r="JD146">
-        <v>1</v>
+        <v>2</v>
       </c>
     </row>
     <row r="147" spans="1:264">
@@ -71978,28 +71978,28 @@
         <v>5</v>
       </c>
       <c r="IW147">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="IX147">
+        <v>1</v>
+      </c>
+      <c r="IY147">
+        <v>1</v>
+      </c>
+      <c r="IZ147">
+        <v>1</v>
+      </c>
+      <c r="JA147">
+        <v>1</v>
+      </c>
+      <c r="JB147">
+        <v>1</v>
+      </c>
+      <c r="JC147">
+        <v>2</v>
+      </c>
+      <c r="JD147">
         <v>5</v>
-      </c>
-      <c r="IY147">
-        <v>1</v>
-      </c>
-      <c r="IZ147">
-        <v>1</v>
-      </c>
-      <c r="JA147">
-        <v>1</v>
-      </c>
-      <c r="JB147">
-        <v>1</v>
-      </c>
-      <c r="JC147">
-        <v>1</v>
-      </c>
-      <c r="JD147">
-        <v>1</v>
       </c>
     </row>
     <row r="148" spans="1:264">
@@ -72478,28 +72478,28 @@
         <v>5</v>
       </c>
       <c r="IW148">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="IX148">
+        <v>1</v>
+      </c>
+      <c r="IY148">
+        <v>1</v>
+      </c>
+      <c r="IZ148">
+        <v>1</v>
+      </c>
+      <c r="JA148">
+        <v>1</v>
+      </c>
+      <c r="JB148">
+        <v>1</v>
+      </c>
+      <c r="JC148">
+        <v>2</v>
+      </c>
+      <c r="JD148">
         <v>7</v>
-      </c>
-      <c r="IY148">
-        <v>1</v>
-      </c>
-      <c r="IZ148">
-        <v>1</v>
-      </c>
-      <c r="JA148">
-        <v>1</v>
-      </c>
-      <c r="JB148">
-        <v>1</v>
-      </c>
-      <c r="JC148">
-        <v>1</v>
-      </c>
-      <c r="JD148">
-        <v>1</v>
       </c>
     </row>
     <row r="149" spans="1:264">
@@ -72981,10 +72981,10 @@
         <v>3</v>
       </c>
       <c r="IW149">
-        <v>3</v>
+        <v>1</v>
       </c>
       <c r="IX149">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="IY149">
         <v>1</v>
@@ -72999,10 +72999,10 @@
         <v>1</v>
       </c>
       <c r="JC149">
-        <v>1</v>
+        <v>3</v>
       </c>
       <c r="JD149">
-        <v>1</v>
+        <v>2</v>
       </c>
     </row>
     <row r="150" spans="1:264">
@@ -73484,10 +73484,10 @@
         <v>3</v>
       </c>
       <c r="IW150">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="IX150">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="IY150">
         <v>1</v>
@@ -73502,10 +73502,10 @@
         <v>1</v>
       </c>
       <c r="JC150">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="JD150">
-        <v>1</v>
+        <v>2</v>
       </c>
     </row>
     <row r="151" spans="1:264">
@@ -73987,10 +73987,10 @@
         <v>3</v>
       </c>
       <c r="IW151">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="IX151">
-        <v>3</v>
+        <v>1</v>
       </c>
       <c r="IY151">
         <v>1</v>
@@ -74005,10 +74005,10 @@
         <v>1</v>
       </c>
       <c r="JC151">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="JD151">
-        <v>1</v>
+        <v>3</v>
       </c>
     </row>
     <row r="152" spans="1:264">
@@ -74417,10 +74417,10 @@
       <c r="IN152">
         <v>2</v>
       </c>
-      <c r="JC152">
-        <v>0</v>
-      </c>
-      <c r="JD152">
+      <c r="JA152">
+        <v>0</v>
+      </c>
+      <c r="JB152">
         <v>0</v>
       </c>
     </row>
@@ -74855,7 +74855,7 @@
         <v>1</v>
       </c>
       <c r="IW153">
-        <v>3</v>
+        <v>1</v>
       </c>
       <c r="IY153">
         <v>1</v>
@@ -74863,11 +74863,11 @@
       <c r="JA153">
         <v>1</v>
       </c>
+      <c r="JB153">
+        <v>0</v>
+      </c>
       <c r="JC153">
-        <v>1</v>
-      </c>
-      <c r="JD153">
-        <v>0</v>
+        <v>3</v>
       </c>
     </row>
     <row r="154" spans="1:264">
@@ -75276,10 +75276,10 @@
       <c r="IN154">
         <v>2</v>
       </c>
-      <c r="JC154">
-        <v>0</v>
-      </c>
-      <c r="JD154">
+      <c r="JA154">
+        <v>0</v>
+      </c>
+      <c r="JB154">
         <v>0</v>
       </c>
     </row>
@@ -75759,28 +75759,28 @@
         <v>1</v>
       </c>
       <c r="IW155">
+        <v>1</v>
+      </c>
+      <c r="IX155">
+        <v>1</v>
+      </c>
+      <c r="IY155">
+        <v>1</v>
+      </c>
+      <c r="IZ155">
+        <v>1</v>
+      </c>
+      <c r="JA155">
+        <v>1</v>
+      </c>
+      <c r="JB155">
+        <v>1</v>
+      </c>
+      <c r="JC155">
         <v>7</v>
       </c>
-      <c r="IX155">
-        <v>2</v>
-      </c>
-      <c r="IY155">
-        <v>1</v>
-      </c>
-      <c r="IZ155">
-        <v>1</v>
-      </c>
-      <c r="JA155">
-        <v>1</v>
-      </c>
-      <c r="JB155">
-        <v>1</v>
-      </c>
-      <c r="JC155">
-        <v>1</v>
-      </c>
       <c r="JD155">
-        <v>1</v>
+        <v>2</v>
       </c>
     </row>
     <row r="156" spans="1:264">
@@ -76262,7 +76262,7 @@
         <v>1</v>
       </c>
       <c r="IX156">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="IY156">
         <v>1</v>
@@ -76280,7 +76280,7 @@
         <v>1</v>
       </c>
       <c r="JD156">
-        <v>1</v>
+        <v>2</v>
       </c>
     </row>
     <row r="157" spans="1:264">
@@ -76710,10 +76710,10 @@
       <c r="IN157">
         <v>2</v>
       </c>
-      <c r="JC157">
-        <v>0</v>
-      </c>
-      <c r="JD157">
+      <c r="JA157">
+        <v>0</v>
+      </c>
+      <c r="JB157">
         <v>0</v>
       </c>
     </row>
@@ -77229,25 +77229,25 @@
         <v>3</v>
       </c>
       <c r="IW158">
+        <v>1</v>
+      </c>
+      <c r="IX158">
+        <v>1</v>
+      </c>
+      <c r="IY158">
+        <v>1</v>
+      </c>
+      <c r="IZ158">
+        <v>1</v>
+      </c>
+      <c r="JA158">
+        <v>1</v>
+      </c>
+      <c r="JB158">
+        <v>1</v>
+      </c>
+      <c r="JC158">
         <v>6</v>
-      </c>
-      <c r="IX158">
-        <v>1</v>
-      </c>
-      <c r="IY158">
-        <v>1</v>
-      </c>
-      <c r="IZ158">
-        <v>1</v>
-      </c>
-      <c r="JA158">
-        <v>1</v>
-      </c>
-      <c r="JB158">
-        <v>1</v>
-      </c>
-      <c r="JC158">
-        <v>1</v>
       </c>
       <c r="JD158">
         <v>1</v>
@@ -77765,10 +77765,10 @@
         <v>3</v>
       </c>
       <c r="IW159">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="IX159">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="IY159">
         <v>1</v>
@@ -77783,10 +77783,10 @@
         <v>1</v>
       </c>
       <c r="JC159">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="JD159">
-        <v>1</v>
+        <v>2</v>
       </c>
     </row>
     <row r="160" spans="1:264">
@@ -78301,28 +78301,28 @@
         <v>3</v>
       </c>
       <c r="IW160">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="IX160">
+        <v>1</v>
+      </c>
+      <c r="IY160">
+        <v>1</v>
+      </c>
+      <c r="IZ160">
+        <v>1</v>
+      </c>
+      <c r="JA160">
+        <v>1</v>
+      </c>
+      <c r="JB160">
+        <v>1</v>
+      </c>
+      <c r="JC160">
+        <v>2</v>
+      </c>
+      <c r="JD160">
         <v>7</v>
-      </c>
-      <c r="IY160">
-        <v>1</v>
-      </c>
-      <c r="IZ160">
-        <v>1</v>
-      </c>
-      <c r="JA160">
-        <v>1</v>
-      </c>
-      <c r="JB160">
-        <v>1</v>
-      </c>
-      <c r="JC160">
-        <v>1</v>
-      </c>
-      <c r="JD160">
-        <v>1</v>
       </c>
     </row>
     <row r="161" spans="1:264">
@@ -78804,10 +78804,10 @@
         <v>3</v>
       </c>
       <c r="IW161">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="IX161">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="IY161">
         <v>1</v>
@@ -78822,10 +78822,10 @@
         <v>1</v>
       </c>
       <c r="JC161">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="JD161">
-        <v>1</v>
+        <v>2</v>
       </c>
     </row>
     <row r="162" spans="1:264">
@@ -79307,28 +79307,28 @@
         <v>3</v>
       </c>
       <c r="IW162">
-        <v>4</v>
+        <v>1</v>
       </c>
       <c r="IX162">
+        <v>1</v>
+      </c>
+      <c r="IY162">
+        <v>1</v>
+      </c>
+      <c r="IZ162">
+        <v>1</v>
+      </c>
+      <c r="JA162">
+        <v>1</v>
+      </c>
+      <c r="JB162">
+        <v>1</v>
+      </c>
+      <c r="JC162">
+        <v>4</v>
+      </c>
+      <c r="JD162">
         <v>5</v>
-      </c>
-      <c r="IY162">
-        <v>1</v>
-      </c>
-      <c r="IZ162">
-        <v>1</v>
-      </c>
-      <c r="JA162">
-        <v>1</v>
-      </c>
-      <c r="JB162">
-        <v>1</v>
-      </c>
-      <c r="JC162">
-        <v>1</v>
-      </c>
-      <c r="JD162">
-        <v>1</v>
       </c>
     </row>
     <row r="163" spans="1:264">
@@ -79810,28 +79810,28 @@
         <v>3</v>
       </c>
       <c r="IW163">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="IX163">
+        <v>1</v>
+      </c>
+      <c r="IY163">
+        <v>1</v>
+      </c>
+      <c r="IZ163">
+        <v>1</v>
+      </c>
+      <c r="JA163">
+        <v>1</v>
+      </c>
+      <c r="JB163">
+        <v>1</v>
+      </c>
+      <c r="JC163">
+        <v>2</v>
+      </c>
+      <c r="JD163">
         <v>7</v>
-      </c>
-      <c r="IY163">
-        <v>1</v>
-      </c>
-      <c r="IZ163">
-        <v>1</v>
-      </c>
-      <c r="JA163">
-        <v>1</v>
-      </c>
-      <c r="JB163">
-        <v>1</v>
-      </c>
-      <c r="JC163">
-        <v>1</v>
-      </c>
-      <c r="JD163">
-        <v>1</v>
       </c>
     </row>
     <row r="164" spans="1:264">
@@ -80261,10 +80261,10 @@
       <c r="IN164">
         <v>2</v>
       </c>
-      <c r="JC164">
-        <v>0</v>
-      </c>
-      <c r="JD164">
+      <c r="JA164">
+        <v>0</v>
+      </c>
+      <c r="JB164">
         <v>0</v>
       </c>
     </row>
@@ -80744,10 +80744,10 @@
         <v>1</v>
       </c>
       <c r="IW165">
-        <v>4</v>
+        <v>1</v>
       </c>
       <c r="IX165">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="IY165">
         <v>1</v>
@@ -80762,10 +80762,10 @@
         <v>1</v>
       </c>
       <c r="JC165">
-        <v>1</v>
+        <v>4</v>
       </c>
       <c r="JD165">
-        <v>1</v>
+        <v>2</v>
       </c>
     </row>
     <row r="166" spans="1:264">
@@ -81244,7 +81244,7 @@
         <v>1</v>
       </c>
       <c r="IW166">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="IX166">
         <v>1</v>
@@ -81262,7 +81262,7 @@
         <v>1</v>
       </c>
       <c r="JC166">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="JD166">
         <v>1</v>
@@ -81744,28 +81744,28 @@
         <v>1</v>
       </c>
       <c r="IW167">
+        <v>1</v>
+      </c>
+      <c r="IX167">
+        <v>1</v>
+      </c>
+      <c r="IY167">
+        <v>1</v>
+      </c>
+      <c r="IZ167">
+        <v>1</v>
+      </c>
+      <c r="JA167">
+        <v>1</v>
+      </c>
+      <c r="JB167">
+        <v>1</v>
+      </c>
+      <c r="JC167">
         <v>6</v>
       </c>
-      <c r="IX167">
+      <c r="JD167">
         <v>5</v>
-      </c>
-      <c r="IY167">
-        <v>1</v>
-      </c>
-      <c r="IZ167">
-        <v>1</v>
-      </c>
-      <c r="JA167">
-        <v>1</v>
-      </c>
-      <c r="JB167">
-        <v>1</v>
-      </c>
-      <c r="JC167">
-        <v>1</v>
-      </c>
-      <c r="JD167">
-        <v>1</v>
       </c>
     </row>
     <row r="168" spans="1:264">
@@ -82244,28 +82244,28 @@
         <v>1</v>
       </c>
       <c r="IW168">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="IX168">
+        <v>1</v>
+      </c>
+      <c r="IY168">
+        <v>1</v>
+      </c>
+      <c r="IZ168">
+        <v>1</v>
+      </c>
+      <c r="JA168">
+        <v>1</v>
+      </c>
+      <c r="JB168">
+        <v>1</v>
+      </c>
+      <c r="JC168">
+        <v>2</v>
+      </c>
+      <c r="JD168">
         <v>5</v>
-      </c>
-      <c r="IY168">
-        <v>1</v>
-      </c>
-      <c r="IZ168">
-        <v>1</v>
-      </c>
-      <c r="JA168">
-        <v>1</v>
-      </c>
-      <c r="JB168">
-        <v>1</v>
-      </c>
-      <c r="JC168">
-        <v>1</v>
-      </c>
-      <c r="JD168">
-        <v>1</v>
       </c>
     </row>
     <row r="169" spans="1:264">
@@ -82744,10 +82744,10 @@
         <v>1</v>
       </c>
       <c r="IW169">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="IX169">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="IY169">
         <v>1</v>
@@ -82762,10 +82762,10 @@
         <v>1</v>
       </c>
       <c r="JC169">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="JD169">
-        <v>1</v>
+        <v>2</v>
       </c>
     </row>
     <row r="170" spans="1:264">
@@ -83244,10 +83244,10 @@
         <v>3</v>
       </c>
       <c r="IW170">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="IX170">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="IY170">
         <v>1</v>
@@ -83262,10 +83262,10 @@
         <v>1</v>
       </c>
       <c r="JC170">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="JD170">
-        <v>1</v>
+        <v>2</v>
       </c>
     </row>
     <row r="171" spans="1:264">
@@ -83744,10 +83744,10 @@
         <v>3</v>
       </c>
       <c r="IW171">
-        <v>3</v>
+        <v>1</v>
       </c>
       <c r="IX171">
-        <v>3</v>
+        <v>1</v>
       </c>
       <c r="IY171">
         <v>1</v>
@@ -83762,10 +83762,10 @@
         <v>1</v>
       </c>
       <c r="JC171">
-        <v>1</v>
+        <v>3</v>
       </c>
       <c r="JD171">
-        <v>1</v>
+        <v>3</v>
       </c>
     </row>
     <row r="172" spans="1:264">
@@ -84220,7 +84220,7 @@
         <v>1</v>
       </c>
       <c r="IW172">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="IY172">
         <v>1</v>
@@ -84228,11 +84228,11 @@
       <c r="JA172">
         <v>1</v>
       </c>
+      <c r="JB172">
+        <v>0</v>
+      </c>
       <c r="JC172">
-        <v>1</v>
-      </c>
-      <c r="JD172">
-        <v>0</v>
+        <v>2</v>
       </c>
     </row>
     <row r="173" spans="1:264">
@@ -84666,7 +84666,7 @@
         <v>3</v>
       </c>
       <c r="IW173">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="IY173">
         <v>1</v>
@@ -84674,11 +84674,11 @@
       <c r="JA173">
         <v>1</v>
       </c>
+      <c r="JB173">
+        <v>0</v>
+      </c>
       <c r="JC173">
-        <v>1</v>
-      </c>
-      <c r="JD173">
-        <v>0</v>
+        <v>2</v>
       </c>
     </row>
     <row r="174" spans="1:264">
@@ -85112,7 +85112,7 @@
         <v>3</v>
       </c>
       <c r="IW174">
-        <v>3</v>
+        <v>1</v>
       </c>
       <c r="IY174">
         <v>1</v>
@@ -85120,11 +85120,11 @@
       <c r="JA174">
         <v>1</v>
       </c>
+      <c r="JB174">
+        <v>0</v>
+      </c>
       <c r="JC174">
-        <v>1</v>
-      </c>
-      <c r="JD174">
-        <v>0</v>
+        <v>3</v>
       </c>
     </row>
     <row r="175" spans="1:264">
@@ -85558,7 +85558,7 @@
         <v>3</v>
       </c>
       <c r="IW175">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="IY175">
         <v>1</v>
@@ -85566,11 +85566,11 @@
       <c r="JA175">
         <v>1</v>
       </c>
+      <c r="JB175">
+        <v>0</v>
+      </c>
       <c r="JC175">
-        <v>1</v>
-      </c>
-      <c r="JD175">
-        <v>0</v>
+        <v>2</v>
       </c>
     </row>
     <row r="176" spans="1:264">
@@ -86049,10 +86049,10 @@
         <v>1</v>
       </c>
       <c r="IW176">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="IX176">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="IY176">
         <v>1</v>
@@ -86067,10 +86067,10 @@
         <v>1</v>
       </c>
       <c r="JC176">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="JD176">
-        <v>1</v>
+        <v>2</v>
       </c>
     </row>
     <row r="177" spans="1:264">
@@ -86525,7 +86525,7 @@
         <v>1</v>
       </c>
       <c r="IW177">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="IY177">
         <v>1</v>
@@ -86533,11 +86533,11 @@
       <c r="JA177">
         <v>1</v>
       </c>
+      <c r="JB177">
+        <v>0</v>
+      </c>
       <c r="JC177">
-        <v>1</v>
-      </c>
-      <c r="JD177">
-        <v>0</v>
+        <v>2</v>
       </c>
     </row>
     <row r="178" spans="1:264">
@@ -87516,10 +87516,10 @@
         <v>1</v>
       </c>
       <c r="IW179">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="IX179">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="IY179">
         <v>1</v>
@@ -87534,10 +87534,10 @@
         <v>1</v>
       </c>
       <c r="JC179">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="JD179">
-        <v>1</v>
+        <v>2</v>
       </c>
     </row>
     <row r="180" spans="1:264">
@@ -88016,28 +88016,28 @@
         <v>1</v>
       </c>
       <c r="IW180">
+        <v>1</v>
+      </c>
+      <c r="IX180">
+        <v>1</v>
+      </c>
+      <c r="IY180">
+        <v>1</v>
+      </c>
+      <c r="IZ180">
+        <v>1</v>
+      </c>
+      <c r="JA180">
+        <v>1</v>
+      </c>
+      <c r="JB180">
+        <v>1</v>
+      </c>
+      <c r="JC180">
         <v>7</v>
       </c>
-      <c r="IX180">
+      <c r="JD180">
         <v>7</v>
-      </c>
-      <c r="IY180">
-        <v>1</v>
-      </c>
-      <c r="IZ180">
-        <v>1</v>
-      </c>
-      <c r="JA180">
-        <v>1</v>
-      </c>
-      <c r="JB180">
-        <v>1</v>
-      </c>
-      <c r="JC180">
-        <v>1</v>
-      </c>
-      <c r="JD180">
-        <v>1</v>
       </c>
     </row>
     <row r="181" spans="1:264">
@@ -88997,11 +88997,11 @@
       <c r="IZ182">
         <v>1</v>
       </c>
+      <c r="JA182">
+        <v>0</v>
+      </c>
       <c r="JB182">
         <v>1</v>
-      </c>
-      <c r="JC182">
-        <v>0</v>
       </c>
       <c r="JD182">
         <v>1</v>
@@ -89459,7 +89459,7 @@
         <v>5</v>
       </c>
       <c r="IW183">
-        <v>4</v>
+        <v>1</v>
       </c>
       <c r="IY183">
         <v>1</v>
@@ -89467,11 +89467,11 @@
       <c r="JA183">
         <v>1</v>
       </c>
+      <c r="JB183">
+        <v>0</v>
+      </c>
       <c r="JC183">
-        <v>1</v>
-      </c>
-      <c r="JD183">
-        <v>0</v>
+        <v>4</v>
       </c>
     </row>
     <row r="184" spans="1:264">
@@ -89926,19 +89926,19 @@
         <v>4</v>
       </c>
       <c r="IX184">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="IZ184">
         <v>1</v>
       </c>
+      <c r="JA184">
+        <v>0</v>
+      </c>
       <c r="JB184">
         <v>1</v>
       </c>
-      <c r="JC184">
-        <v>0</v>
-      </c>
       <c r="JD184">
-        <v>1</v>
+        <v>2</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Renumber individual_type to 1-6, remove Type 4 立场坚持者
</commit_message>
<xml_diff>
--- a/dataset2026.xlsx
+++ b/dataset2026.xlsx
@@ -3342,7 +3342,7 @@
         <v>0</v>
       </c>
       <c r="JC2">
-        <v>6</v>
+        <v>5</v>
       </c>
     </row>
     <row r="3" spans="1:264">
@@ -5117,7 +5117,7 @@
         <v>1</v>
       </c>
       <c r="JD6">
-        <v>7</v>
+        <v>6</v>
       </c>
     </row>
     <row r="7" spans="1:264">
@@ -5994,7 +5994,7 @@
         <v>1</v>
       </c>
       <c r="JD8">
-        <v>7</v>
+        <v>6</v>
       </c>
     </row>
     <row r="9" spans="1:264">
@@ -6449,7 +6449,7 @@
         <v>1</v>
       </c>
       <c r="JD9">
-        <v>6</v>
+        <v>5</v>
       </c>
     </row>
     <row r="10" spans="1:264">
@@ -6904,7 +6904,7 @@
         <v>1</v>
       </c>
       <c r="JD10">
-        <v>6</v>
+        <v>5</v>
       </c>
     </row>
     <row r="11" spans="1:264">
@@ -8754,7 +8754,7 @@
         <v>2</v>
       </c>
       <c r="JD14">
-        <v>7</v>
+        <v>6</v>
       </c>
     </row>
     <row r="15" spans="1:264">
@@ -12690,7 +12690,7 @@
         <v>0</v>
       </c>
       <c r="JC23">
-        <v>4</v>
+        <v>5</v>
       </c>
     </row>
     <row r="24" spans="1:264">
@@ -13588,7 +13588,7 @@
         <v>0</v>
       </c>
       <c r="JC25">
-        <v>7</v>
+        <v>6</v>
       </c>
     </row>
     <row r="26" spans="1:264">
@@ -15600,7 +15600,7 @@
         <v>1</v>
       </c>
       <c r="JD29">
-        <v>7</v>
+        <v>6</v>
       </c>
     </row>
     <row r="30" spans="1:264">
@@ -16103,7 +16103,7 @@
         <v>2</v>
       </c>
       <c r="JD30">
-        <v>7</v>
+        <v>6</v>
       </c>
     </row>
     <row r="31" spans="1:264">
@@ -16603,10 +16603,10 @@
         <v>1</v>
       </c>
       <c r="JC31">
-        <v>6</v>
+        <v>5</v>
       </c>
       <c r="JD31">
-        <v>6</v>
+        <v>5</v>
       </c>
     </row>
     <row r="32" spans="1:264">
@@ -17106,10 +17106,10 @@
         <v>1</v>
       </c>
       <c r="JC32">
-        <v>4</v>
+        <v>1</v>
       </c>
       <c r="JD32">
-        <v>6</v>
+        <v>5</v>
       </c>
     </row>
     <row r="33" spans="1:264">
@@ -18046,7 +18046,7 @@
         <v>1</v>
       </c>
       <c r="JC34">
-        <v>4</v>
+        <v>6</v>
       </c>
       <c r="JD34">
         <v>2</v>
@@ -21698,10 +21698,10 @@
         <v>1</v>
       </c>
       <c r="JC42">
-        <v>4</v>
+        <v>1</v>
       </c>
       <c r="JD42">
-        <v>5</v>
+        <v>4</v>
       </c>
     </row>
     <row r="43" spans="1:264">
@@ -23677,7 +23677,7 @@
         <v>1</v>
       </c>
       <c r="JC46">
-        <v>4</v>
+        <v>1</v>
       </c>
       <c r="JD46">
         <v>2</v>
@@ -24183,7 +24183,7 @@
         <v>3</v>
       </c>
       <c r="JD47">
-        <v>5</v>
+        <v>4</v>
       </c>
     </row>
     <row r="48" spans="1:264">
@@ -26665,10 +26665,10 @@
         <v>1</v>
       </c>
       <c r="JC52">
-        <v>4</v>
+        <v>1</v>
       </c>
       <c r="JD52">
-        <v>7</v>
+        <v>6</v>
       </c>
     </row>
     <row r="53" spans="1:264">
@@ -27114,7 +27114,7 @@
         <v>0</v>
       </c>
       <c r="JC53">
-        <v>7</v>
+        <v>6</v>
       </c>
     </row>
     <row r="54" spans="1:264">
@@ -31970,10 +31970,10 @@
         <v>1</v>
       </c>
       <c r="JC63">
-        <v>6</v>
+        <v>5</v>
       </c>
       <c r="JD63">
-        <v>6</v>
+        <v>5</v>
       </c>
     </row>
     <row r="64" spans="1:264">
@@ -32970,10 +32970,10 @@
         <v>1</v>
       </c>
       <c r="JC65">
-        <v>4</v>
+        <v>5</v>
       </c>
       <c r="JD65">
-        <v>7</v>
+        <v>6</v>
       </c>
     </row>
     <row r="66" spans="1:264">
@@ -33970,7 +33970,7 @@
         <v>1</v>
       </c>
       <c r="JC67">
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="JD67">
         <v>1</v>
@@ -34473,7 +34473,7 @@
         <v>1</v>
       </c>
       <c r="JD68">
-        <v>7</v>
+        <v>6</v>
       </c>
     </row>
     <row r="69" spans="1:264">
@@ -35937,7 +35937,7 @@
         <v>1</v>
       </c>
       <c r="JC71">
-        <v>7</v>
+        <v>6</v>
       </c>
       <c r="JD71">
         <v>2</v>
@@ -40113,7 +40113,7 @@
         <v>2</v>
       </c>
       <c r="JD80">
-        <v>7</v>
+        <v>6</v>
       </c>
     </row>
     <row r="81" spans="1:264">
@@ -40613,7 +40613,7 @@
         <v>2</v>
       </c>
       <c r="JD81">
-        <v>6</v>
+        <v>5</v>
       </c>
     </row>
     <row r="82" spans="1:264">
@@ -41110,7 +41110,7 @@
         <v>1</v>
       </c>
       <c r="JC82">
-        <v>4</v>
+        <v>5</v>
       </c>
       <c r="JD82">
         <v>2</v>
@@ -43199,7 +43199,7 @@
         <v>0</v>
       </c>
       <c r="JC87">
-        <v>7</v>
+        <v>6</v>
       </c>
     </row>
     <row r="88" spans="1:264">
@@ -44112,7 +44112,7 @@
         <v>1</v>
       </c>
       <c r="JD89">
-        <v>7</v>
+        <v>6</v>
       </c>
     </row>
     <row r="90" spans="1:264">
@@ -47624,7 +47624,7 @@
         <v>1</v>
       </c>
       <c r="JC96">
-        <v>4</v>
+        <v>1</v>
       </c>
       <c r="JD96">
         <v>1</v>
@@ -48127,7 +48127,7 @@
         <v>1</v>
       </c>
       <c r="JC97">
-        <v>4</v>
+        <v>5</v>
       </c>
       <c r="JD97">
         <v>2</v>
@@ -49028,7 +49028,7 @@
         <v>0</v>
       </c>
       <c r="JC99">
-        <v>6</v>
+        <v>5</v>
       </c>
     </row>
     <row r="100" spans="1:264">
@@ -50480,7 +50480,7 @@
         <v>1</v>
       </c>
       <c r="JC102">
-        <v>4</v>
+        <v>5</v>
       </c>
       <c r="JD102">
         <v>2</v>
@@ -53498,7 +53498,7 @@
         <v>1</v>
       </c>
       <c r="JC108">
-        <v>4</v>
+        <v>1</v>
       </c>
       <c r="JD108">
         <v>2</v>
@@ -54001,7 +54001,7 @@
         <v>1</v>
       </c>
       <c r="JC109">
-        <v>4</v>
+        <v>6</v>
       </c>
       <c r="JD109">
         <v>2</v>
@@ -59731,10 +59731,10 @@
         <v>1</v>
       </c>
       <c r="JC121">
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="JD121">
-        <v>5</v>
+        <v>4</v>
       </c>
     </row>
     <row r="122" spans="1:264">
@@ -60632,7 +60632,7 @@
         <v>0</v>
       </c>
       <c r="JC123">
-        <v>4</v>
+        <v>6</v>
       </c>
     </row>
     <row r="124" spans="1:264">
@@ -61584,7 +61584,7 @@
         <v>2</v>
       </c>
       <c r="JD125">
-        <v>7</v>
+        <v>6</v>
       </c>
     </row>
     <row r="126" spans="1:264">
@@ -62084,7 +62084,7 @@
         <v>1</v>
       </c>
       <c r="JC126">
-        <v>4</v>
+        <v>1</v>
       </c>
       <c r="JD126">
         <v>1</v>
@@ -63560,7 +63560,7 @@
         <v>1</v>
       </c>
       <c r="JC129">
-        <v>4</v>
+        <v>6</v>
       </c>
       <c r="JD129">
         <v>2</v>
@@ -65431,7 +65431,7 @@
         <v>0</v>
       </c>
       <c r="JC133">
-        <v>7</v>
+        <v>6</v>
       </c>
     </row>
     <row r="134" spans="1:264">
@@ -65886,7 +65886,7 @@
         <v>1</v>
       </c>
       <c r="JD134">
-        <v>7</v>
+        <v>6</v>
       </c>
     </row>
     <row r="135" spans="1:264">
@@ -69499,7 +69499,7 @@
         <v>2</v>
       </c>
       <c r="JD142">
-        <v>7</v>
+        <v>6</v>
       </c>
     </row>
     <row r="143" spans="1:264">
@@ -69996,10 +69996,10 @@
         <v>1</v>
       </c>
       <c r="JC143">
-        <v>4</v>
+        <v>1</v>
       </c>
       <c r="JD143">
-        <v>5</v>
+        <v>4</v>
       </c>
     </row>
     <row r="144" spans="1:264">
@@ -70499,7 +70499,7 @@
         <v>1</v>
       </c>
       <c r="JD144">
-        <v>6</v>
+        <v>5</v>
       </c>
     </row>
     <row r="145" spans="1:264">
@@ -70999,7 +70999,7 @@
         <v>2</v>
       </c>
       <c r="JD145">
-        <v>7</v>
+        <v>6</v>
       </c>
     </row>
     <row r="146" spans="1:264">
@@ -71999,7 +71999,7 @@
         <v>2</v>
       </c>
       <c r="JD147">
-        <v>5</v>
+        <v>4</v>
       </c>
     </row>
     <row r="148" spans="1:264">
@@ -72499,7 +72499,7 @@
         <v>2</v>
       </c>
       <c r="JD148">
-        <v>7</v>
+        <v>6</v>
       </c>
     </row>
     <row r="149" spans="1:264">
@@ -75777,7 +75777,7 @@
         <v>1</v>
       </c>
       <c r="JC155">
-        <v>7</v>
+        <v>6</v>
       </c>
       <c r="JD155">
         <v>2</v>
@@ -77247,7 +77247,7 @@
         <v>1</v>
       </c>
       <c r="JC158">
-        <v>6</v>
+        <v>5</v>
       </c>
       <c r="JD158">
         <v>1</v>
@@ -78322,7 +78322,7 @@
         <v>2</v>
       </c>
       <c r="JD160">
-        <v>7</v>
+        <v>6</v>
       </c>
     </row>
     <row r="161" spans="1:264">
@@ -79325,10 +79325,10 @@
         <v>1</v>
       </c>
       <c r="JC162">
-        <v>4</v>
+        <v>6</v>
       </c>
       <c r="JD162">
-        <v>5</v>
+        <v>4</v>
       </c>
     </row>
     <row r="163" spans="1:264">
@@ -79831,7 +79831,7 @@
         <v>2</v>
       </c>
       <c r="JD163">
-        <v>7</v>
+        <v>6</v>
       </c>
     </row>
     <row r="164" spans="1:264">
@@ -80762,7 +80762,7 @@
         <v>1</v>
       </c>
       <c r="JC165">
-        <v>4</v>
+        <v>1</v>
       </c>
       <c r="JD165">
         <v>2</v>
@@ -81762,10 +81762,10 @@
         <v>1</v>
       </c>
       <c r="JC167">
-        <v>6</v>
+        <v>5</v>
       </c>
       <c r="JD167">
-        <v>5</v>
+        <v>4</v>
       </c>
     </row>
     <row r="168" spans="1:264">
@@ -82265,7 +82265,7 @@
         <v>2</v>
       </c>
       <c r="JD168">
-        <v>5</v>
+        <v>4</v>
       </c>
     </row>
     <row r="169" spans="1:264">
@@ -88034,10 +88034,10 @@
         <v>1</v>
       </c>
       <c r="JC180">
-        <v>7</v>
+        <v>6</v>
       </c>
       <c r="JD180">
-        <v>7</v>
+        <v>6</v>
       </c>
     </row>
     <row r="181" spans="1:264">
@@ -89471,7 +89471,7 @@
         <v>0</v>
       </c>
       <c r="JC183">
-        <v>4</v>
+        <v>1</v>
       </c>
     </row>
     <row r="184" spans="1:264">

</xml_diff>

<commit_message>
Final 5 individual types (1-5), remove bystander category
</commit_message>
<xml_diff>
--- a/dataset2026.xlsx
+++ b/dataset2026.xlsx
@@ -3342,7 +3342,7 @@
         <v>0</v>
       </c>
       <c r="JC2">
-        <v>5</v>
+        <v>4</v>
       </c>
     </row>
     <row r="3" spans="1:264">
@@ -5117,7 +5117,7 @@
         <v>1</v>
       </c>
       <c r="JD6">
-        <v>6</v>
+        <v>5</v>
       </c>
     </row>
     <row r="7" spans="1:264">
@@ -5994,7 +5994,7 @@
         <v>1</v>
       </c>
       <c r="JD8">
-        <v>6</v>
+        <v>5</v>
       </c>
     </row>
     <row r="9" spans="1:264">
@@ -6449,7 +6449,7 @@
         <v>1</v>
       </c>
       <c r="JD9">
-        <v>5</v>
+        <v>4</v>
       </c>
     </row>
     <row r="10" spans="1:264">
@@ -6904,7 +6904,7 @@
         <v>1</v>
       </c>
       <c r="JD10">
-        <v>5</v>
+        <v>4</v>
       </c>
     </row>
     <row r="11" spans="1:264">
@@ -8754,7 +8754,7 @@
         <v>2</v>
       </c>
       <c r="JD14">
-        <v>6</v>
+        <v>5</v>
       </c>
     </row>
     <row r="15" spans="1:264">
@@ -12690,7 +12690,7 @@
         <v>0</v>
       </c>
       <c r="JC23">
-        <v>5</v>
+        <v>4</v>
       </c>
     </row>
     <row r="24" spans="1:264">
@@ -13588,7 +13588,7 @@
         <v>0</v>
       </c>
       <c r="JC25">
-        <v>6</v>
+        <v>5</v>
       </c>
     </row>
     <row r="26" spans="1:264">
@@ -15600,7 +15600,7 @@
         <v>1</v>
       </c>
       <c r="JD29">
-        <v>6</v>
+        <v>5</v>
       </c>
     </row>
     <row r="30" spans="1:264">
@@ -16103,7 +16103,7 @@
         <v>2</v>
       </c>
       <c r="JD30">
-        <v>6</v>
+        <v>5</v>
       </c>
     </row>
     <row r="31" spans="1:264">
@@ -16603,10 +16603,10 @@
         <v>1</v>
       </c>
       <c r="JC31">
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="JD31">
-        <v>5</v>
+        <v>4</v>
       </c>
     </row>
     <row r="32" spans="1:264">
@@ -17109,7 +17109,7 @@
         <v>1</v>
       </c>
       <c r="JD32">
-        <v>5</v>
+        <v>4</v>
       </c>
     </row>
     <row r="33" spans="1:264">
@@ -18046,7 +18046,7 @@
         <v>1</v>
       </c>
       <c r="JC34">
-        <v>6</v>
+        <v>5</v>
       </c>
       <c r="JD34">
         <v>2</v>
@@ -21701,7 +21701,7 @@
         <v>1</v>
       </c>
       <c r="JD42">
-        <v>4</v>
+        <v>2</v>
       </c>
     </row>
     <row r="43" spans="1:264">
@@ -24183,7 +24183,7 @@
         <v>3</v>
       </c>
       <c r="JD47">
-        <v>4</v>
+        <v>2</v>
       </c>
     </row>
     <row r="48" spans="1:264">
@@ -26668,7 +26668,7 @@
         <v>1</v>
       </c>
       <c r="JD52">
-        <v>6</v>
+        <v>5</v>
       </c>
     </row>
     <row r="53" spans="1:264">
@@ -27114,7 +27114,7 @@
         <v>0</v>
       </c>
       <c r="JC53">
-        <v>6</v>
+        <v>5</v>
       </c>
     </row>
     <row r="54" spans="1:264">
@@ -31970,10 +31970,10 @@
         <v>1</v>
       </c>
       <c r="JC63">
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="JD63">
-        <v>5</v>
+        <v>4</v>
       </c>
     </row>
     <row r="64" spans="1:264">
@@ -32970,10 +32970,10 @@
         <v>1</v>
       </c>
       <c r="JC65">
+        <v>4</v>
+      </c>
+      <c r="JD65">
         <v>5</v>
-      </c>
-      <c r="JD65">
-        <v>6</v>
       </c>
     </row>
     <row r="66" spans="1:264">
@@ -33970,7 +33970,7 @@
         <v>1</v>
       </c>
       <c r="JC67">
-        <v>4</v>
+        <v>2</v>
       </c>
       <c r="JD67">
         <v>1</v>
@@ -34473,7 +34473,7 @@
         <v>1</v>
       </c>
       <c r="JD68">
-        <v>6</v>
+        <v>5</v>
       </c>
     </row>
     <row r="69" spans="1:264">
@@ -35937,7 +35937,7 @@
         <v>1</v>
       </c>
       <c r="JC71">
-        <v>6</v>
+        <v>5</v>
       </c>
       <c r="JD71">
         <v>2</v>
@@ -40113,7 +40113,7 @@
         <v>2</v>
       </c>
       <c r="JD80">
-        <v>6</v>
+        <v>5</v>
       </c>
     </row>
     <row r="81" spans="1:264">
@@ -40613,7 +40613,7 @@
         <v>2</v>
       </c>
       <c r="JD81">
-        <v>5</v>
+        <v>4</v>
       </c>
     </row>
     <row r="82" spans="1:264">
@@ -41110,7 +41110,7 @@
         <v>1</v>
       </c>
       <c r="JC82">
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="JD82">
         <v>2</v>
@@ -43199,7 +43199,7 @@
         <v>0</v>
       </c>
       <c r="JC87">
-        <v>6</v>
+        <v>5</v>
       </c>
     </row>
     <row r="88" spans="1:264">
@@ -44112,7 +44112,7 @@
         <v>1</v>
       </c>
       <c r="JD89">
-        <v>6</v>
+        <v>5</v>
       </c>
     </row>
     <row r="90" spans="1:264">
@@ -48127,7 +48127,7 @@
         <v>1</v>
       </c>
       <c r="JC97">
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="JD97">
         <v>2</v>
@@ -49028,7 +49028,7 @@
         <v>0</v>
       </c>
       <c r="JC99">
-        <v>5</v>
+        <v>4</v>
       </c>
     </row>
     <row r="100" spans="1:264">
@@ -50480,7 +50480,7 @@
         <v>1</v>
       </c>
       <c r="JC102">
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="JD102">
         <v>2</v>
@@ -54001,7 +54001,7 @@
         <v>1</v>
       </c>
       <c r="JC109">
-        <v>6</v>
+        <v>5</v>
       </c>
       <c r="JD109">
         <v>2</v>
@@ -59731,10 +59731,10 @@
         <v>1</v>
       </c>
       <c r="JC121">
-        <v>4</v>
+        <v>2</v>
       </c>
       <c r="JD121">
-        <v>4</v>
+        <v>2</v>
       </c>
     </row>
     <row r="122" spans="1:264">
@@ -60632,7 +60632,7 @@
         <v>0</v>
       </c>
       <c r="JC123">
-        <v>6</v>
+        <v>5</v>
       </c>
     </row>
     <row r="124" spans="1:264">
@@ -61584,7 +61584,7 @@
         <v>2</v>
       </c>
       <c r="JD125">
-        <v>6</v>
+        <v>5</v>
       </c>
     </row>
     <row r="126" spans="1:264">
@@ -63560,7 +63560,7 @@
         <v>1</v>
       </c>
       <c r="JC129">
-        <v>6</v>
+        <v>5</v>
       </c>
       <c r="JD129">
         <v>2</v>
@@ -65431,7 +65431,7 @@
         <v>0</v>
       </c>
       <c r="JC133">
-        <v>6</v>
+        <v>5</v>
       </c>
     </row>
     <row r="134" spans="1:264">
@@ -65886,7 +65886,7 @@
         <v>1</v>
       </c>
       <c r="JD134">
-        <v>6</v>
+        <v>5</v>
       </c>
     </row>
     <row r="135" spans="1:264">
@@ -69499,7 +69499,7 @@
         <v>2</v>
       </c>
       <c r="JD142">
-        <v>6</v>
+        <v>5</v>
       </c>
     </row>
     <row r="143" spans="1:264">
@@ -69999,7 +69999,7 @@
         <v>1</v>
       </c>
       <c r="JD143">
-        <v>4</v>
+        <v>2</v>
       </c>
     </row>
     <row r="144" spans="1:264">
@@ -70499,7 +70499,7 @@
         <v>1</v>
       </c>
       <c r="JD144">
-        <v>5</v>
+        <v>4</v>
       </c>
     </row>
     <row r="145" spans="1:264">
@@ -70999,7 +70999,7 @@
         <v>2</v>
       </c>
       <c r="JD145">
-        <v>6</v>
+        <v>5</v>
       </c>
     </row>
     <row r="146" spans="1:264">
@@ -71999,7 +71999,7 @@
         <v>2</v>
       </c>
       <c r="JD147">
-        <v>4</v>
+        <v>2</v>
       </c>
     </row>
     <row r="148" spans="1:264">
@@ -72499,7 +72499,7 @@
         <v>2</v>
       </c>
       <c r="JD148">
-        <v>6</v>
+        <v>5</v>
       </c>
     </row>
     <row r="149" spans="1:264">
@@ -75777,7 +75777,7 @@
         <v>1</v>
       </c>
       <c r="JC155">
-        <v>6</v>
+        <v>5</v>
       </c>
       <c r="JD155">
         <v>2</v>
@@ -77247,7 +77247,7 @@
         <v>1</v>
       </c>
       <c r="JC158">
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="JD158">
         <v>1</v>
@@ -78322,7 +78322,7 @@
         <v>2</v>
       </c>
       <c r="JD160">
-        <v>6</v>
+        <v>5</v>
       </c>
     </row>
     <row r="161" spans="1:264">
@@ -79325,10 +79325,10 @@
         <v>1</v>
       </c>
       <c r="JC162">
-        <v>6</v>
+        <v>5</v>
       </c>
       <c r="JD162">
-        <v>4</v>
+        <v>3</v>
       </c>
     </row>
     <row r="163" spans="1:264">
@@ -79831,7 +79831,7 @@
         <v>2</v>
       </c>
       <c r="JD163">
-        <v>6</v>
+        <v>5</v>
       </c>
     </row>
     <row r="164" spans="1:264">
@@ -81762,7 +81762,7 @@
         <v>1</v>
       </c>
       <c r="JC167">
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="JD167">
         <v>4</v>
@@ -82265,7 +82265,7 @@
         <v>2</v>
       </c>
       <c r="JD168">
-        <v>4</v>
+        <v>2</v>
       </c>
     </row>
     <row r="169" spans="1:264">
@@ -88034,10 +88034,10 @@
         <v>1</v>
       </c>
       <c r="JC180">
-        <v>6</v>
+        <v>5</v>
       </c>
       <c r="JD180">
-        <v>6</v>
+        <v>5</v>
       </c>
     </row>
     <row r="181" spans="1:264">

</xml_diff>